<commit_message>
feat(F-NAR-009): ramifiées AUT-003, 004, 007, 008
Ouvertures du monde, 86 passages, texte seulement.
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-AUT-003.xlsx
+++ b/stories/arbres/TREE-AUT-003.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -552,7 +552,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Retrouver ses affaires avant de partir — dans le salon</t>
+          <t>La goutte sur la vitre</t>
         </is>
       </c>
     </row>
@@ -843,6 +843,18 @@
       <c r="B30" t="inlineStr">
         <is>
           <t>voix-roles-v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>fil_rouge</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Nino va au parc avec papa et maman. Une goutte brille encore sur la vitre. Ses affaires sont dans la maison. Il les reprend avant de partir.</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1197,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Maya est dans le salon, avec maman. Papa cherche les chaussures. Bientôt on part. Il y a un seau, un manteau, un doudou. On va reprendre ses affaires avant de partir.</t>
+          <t>Une goutte glisse sur la vitre. Elle laisse une trace brillante. Le salon sent le cacao. Un carré de soleil pose sur le tapis. Le tapis est chaud, juste là. Les chaussons de Nino attendent près du canapé. Papa ouvre le placard de l'entrée. Les crochets font un petit cliquetis. Nino, on sort bientôt. On va au parc, avec papa. J'arrive, maman. Une cuillère tinte dans une tasse. En ce moment, Nino est dans le salon. Il voit le seau près de la porte. Le seau est bleu, un peu sablé. Le manteau est sur une chaise. Le doudou cache son oreille sous un coussin. Tes affaires sont prêtes, Nino ? Je sais plus, papa. On les reprend ensemble. Nino pose un pied sur le tapis chaud. Il regarde la cuisine. Il regarde la porte du jardin. Il regarde le couloir de la chambre.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1325,8 +1337,30 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Maya est dans le salon, avec maman. Papa cherche les chaussures. Bientôt on part. Il y a un seau, un manteau, un doudou.
-maman|On va reprendre ses affaires avant de partir.</t>
+          <t>narrateur|Une goutte glisse sur la vitre.
+narrateur|Elle laisse une trace brillante.
+narrateur|Le salon sent le cacao.
+narrateur|Un carré de soleil pose sur le tapis.
+narrateur|Le tapis est chaud, juste là.
+narrateur|Les chaussons de Nino attendent près du canapé.
+narrateur|Papa ouvre le placard de l'entrée.
+narrateur|Les crochets font un petit cliquetis.
+maman|Nino, on sort bientôt.
+maman|On va au parc, avec papa.
+enfant-m|J'arrive, maman.
+narrateur|Une cuillère tinte dans une tasse.
+narrateur|En ce moment, Nino est dans le salon.
+narrateur|Il voit le seau près de la porte.
+narrateur|Le seau est bleu, un peu sablé.
+narrateur|Le manteau est sur une chaise.
+narrateur|Le doudou cache son oreille sous un coussin.
+papa|Tes affaires sont prêtes, Nino ?
+enfant-m|Je sais plus, papa.
+papa|On les reprend ensemble.
+narrateur|Nino pose un pied sur le tapis chaud.
+narrateur|Il regarde la cuisine.
+narrateur|Il regarde la porte du jardin.
+narrateur|Il regarde le couloir de la chambre.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr"/>
@@ -1354,7 +1388,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre la cuisine, le jardin, ou la chambre.</t>
+          <t>Nino cherche où, d'abord ? La cuisine, le jardin, ou la chambre ? Tu choisis, Nino.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1518,7 +1552,9 @@
       <c r="AV3" s="2" t="inlineStr"/>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre la cuisine, le jardin, ou la chambre.</t>
+          <t>narrateur|Nino cherche où, d'abord ?
+papa|La cuisine, le jardin, ou la chambre ?
+maman|Tu choisis, Nino.</t>
         </is>
       </c>
       <c r="AX3" t="inlineStr"/>
@@ -1546,7 +1582,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Maya va dans la cuisine. Elle cherche. Elle reprend ses affaires avant de partir. Un gant est sur la table. Prends-le. Maya le met avec le reste.</t>
+          <t>Nino pousse la porte de la cuisine. Ça sent le cacao, plus fort. La table est un peu collante. Un gant rouge est près de la tasse. Le gant est sur la table. Tu le prends, Nino ? Oui. Je le prends. Nino prend le gant. Il est doux et encore un peu chaud. Il le serre contre lui. Bravo, Nino. Tu reprends tes affaires, avant de partir. La table est vide, maintenant. On cherche aussi le seau et le manteau. D'accord, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1686,12 +1722,28 @@
       <c r="AV4" s="2" t="inlineStr"/>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Maya va dans la cuisine. Elle cherche. Elle reprend ses affaires avant de partir. Un gant est sur la table.
-maman|Prends-le.
-narrateur|Maya le met avec le reste.</t>
-        </is>
-      </c>
-      <c r="AX4" t="inlineStr"/>
+          <t>narrateur|Nino pousse la porte de la cuisine.
+narrateur|Ça sent le cacao, plus fort.
+narrateur|La table est un peu collante.
+narrateur|Un gant rouge est près de la tasse.
+maman|Le gant est sur la table.
+maman|Tu le prends, Nino ?
+enfant-m|Oui. Je le prends.
+narrateur|Nino prend le gant.
+narrateur|Il est doux et encore un peu chaud.
+narrateur|Il le serre contre lui.
+papa|Bravo, Nino.
+papa|Tu reprends tes affaires, avant de partir.
+narrateur|La table est vide, maintenant.
+maman|On cherche aussi le seau et le manteau.
+enfant-m|D'accord, maman.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>chaise</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1716,7 +1768,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Avant de partir, on reprend ses affaires ?</t>
+          <t>Avant de partir, Nino reprend ses affaires ?</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1876,7 +1928,7 @@
       </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Avant de partir, on reprend ses affaires ?</t>
+          <t>narrateur|Avant de partir, Nino reprend ses affaires ?</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr"/>
@@ -1904,7 +1956,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Oui. On va reprendre ses affaires avant de partir. Maya respire. Maman est là. On va reprendre ses affaires avant de partir.</t>
+          <t>Oui. Nino a repris le gant. Il le tient bien. Bravo. C'est du bon travail. Avant de partir, on reprend ses affaires. Tu as le gant, Nino ? Oui, papa. Nino souffle un peu. Il est prêt à chercher encore.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -2048,7 +2100,15 @@
       </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Oui. On va reprendre ses affaires avant de partir. Maya respire. Maman est là. On va reprendre ses affaires avant de partir.</t>
+          <t>narrateur|Oui.
+narrateur|Nino a repris le gant.
+narrateur|Il le tient bien.
+maman|Bravo. C'est du bon travail.
+maman|Avant de partir, on reprend ses affaires.
+papa|Tu as le gant, Nino ?
+enfant-m|Oui, papa.
+narrateur|Nino souffle un peu.
+narrateur|Il est prêt à chercher encore.</t>
         </is>
       </c>
       <c r="AX6" t="inlineStr"/>
@@ -2076,7 +2136,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre le ballon rouge, le seau bleu, ou le doudou.</t>
+          <t>Il reste un objet, dans la cuisine. Le ballon rouge, le seau bleu, ou le doudou ?</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -2240,7 +2300,8 @@
       <c r="AV7" s="2" t="inlineStr"/>
       <c r="AW7" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre le ballon rouge, le seau bleu, ou le doudou.</t>
+          <t>narrateur|Il reste un objet, dans la cuisine.
+maman|Le ballon rouge, le seau bleu, ou le doudou ?</t>
         </is>
       </c>
       <c r="AX7" t="inlineStr"/>
@@ -2268,7 +2329,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Maya trouve le ballon rouge. Elle reprend ses affaires avant de partir. Elle le met près de la porte. Encore le manteau. Maman montre le geste, lentement. On va reprendre ses affaires avant de partir.</t>
+          <t>Nino est encore dans la cuisine. Ça sent encore le cacao. Le ballon rouge est sous la table. Il a une miette collée dessus. Le ballon, Nino. Tu le reprends ? Oui. Le ballon rouge. Nino le fait rouler tout doux, jusqu'à lui. Bravo. Tu le mets près de la porte. Le ballon est lisse, un peu poussiéreux. Nino pose le ballon rouge près de la porte. Le carrelage est un peu froid. Nino souffle sur le ballon. Un peu de poussière part. Tu as repris le ballon, avant de partir. Il vient au parc. On reprend ses affaires, avant de partir.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -2408,8 +2469,21 @@
       <c r="AV8" s="2" t="inlineStr"/>
       <c r="AW8" t="inlineStr">
         <is>
-          <t>narrateur|Maya trouve le ballon rouge. Elle reprend ses affaires avant de partir. Elle le met près de la porte.
-maman|Encore le manteau. Maman montre le geste, lentement. On va reprendre ses affaires avant de partir.</t>
+          <t>narrateur|Nino est encore dans la cuisine.
+narrateur|Ça sent encore le cacao.
+narrateur|Le ballon rouge est sous la table.
+narrateur|Il a une miette collée dessus.
+maman|Le ballon, Nino. Tu le reprends ?
+enfant-m|Oui. Le ballon rouge.
+narrateur|Nino le fait rouler tout doux, jusqu'à lui.
+papa|Bravo. Tu le mets près de la porte.
+narrateur|Le ballon est lisse, un peu poussiéreux.
+narrateur|Nino pose le ballon rouge près de la porte.
+narrateur|Le carrelage est un peu froid.
+narrateur|Nino souffle sur le ballon. Un peu de poussière part.
+papa|Tu as repris le ballon, avant de partir.
+enfant-m|Il vient au parc.
+maman|On reprend ses affaires, avant de partir.</t>
         </is>
       </c>
       <c r="AX8" t="inlineStr"/>
@@ -2437,7 +2511,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre Tom, Léa, ou Sami.</t>
+          <t>Il reste une chose, pour sortir. Le sac, le manteau, ou les chaussures ? Tu choisis, Nino.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -2605,7 +2679,9 @@
       </c>
       <c r="AW9" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre Tom, Léa, ou Sami.</t>
+          <t>narrateur|Il reste une chose, pour sortir.
+papa|Le sac, le manteau, ou les chaussures ?
+maman|Tu choisis, Nino.</t>
         </is>
       </c>
       <c r="AX9" t="inlineStr"/>
@@ -2633,7 +2709,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Maya a choisi la cuisine. Puis le ballon rouge. Puis Tom. Une feuille tombe. Maya serre la main de maman. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>Nino a cherché la cuisine. Il a repris le ballon rouge. Maintenant, le sac. Une feuille collée à la vitre se détache. Nino ouvre le sac. Il y glisse ce qu'il a repris. Tout est près de la porte. Bravo, Nino. Tes affaires sont près de la porte. J'ai le sac ! Nino reprend ses affaires, avant de partir. On a le seau. On a le manteau. On les prend. On peut sortir. Nino serre ce qu'il tient. Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -2773,10 +2849,26 @@
       <c r="AV10" s="2" t="inlineStr"/>
       <c r="AW10" t="inlineStr">
         <is>
-          <t>narrateur|Maya a choisi la cuisine. Puis le ballon rouge. Puis Tom. Une feuille tombe. Maya serre la main de maman. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
-        </is>
-      </c>
-      <c r="AX10" t="inlineStr"/>
+          <t>narrateur|Nino a cherché la cuisine.
+narrateur|Il a repris le ballon rouge.
+narrateur|Maintenant, le sac.
+narrateur|Une feuille collée à la vitre se détache.
+narrateur|Nino ouvre le sac. Il y glisse ce qu'il a repris.
+narrateur|Tout est près de la porte.
+papa|Bravo, Nino. Tes affaires sont près de la porte.
+enfant-m|J'ai le sac !
+narrateur|Nino reprend ses affaires, avant de partir.
+maman|On a le seau. On a le manteau.
+papa|On les prend. On peut sortir.
+narrateur|Nino serre ce qu'il tient.
+enfant-m|Merci, maman. Merci, papa.</t>
+        </is>
+      </c>
+      <c r="AX10" t="inlineStr">
+        <is>
+          <t>porte</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2801,7 +2893,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>L'air du parc sent l'herbe coupée. Nino a repris ses affaires. C'était avant de partir. Bravo, Nino. Tu as fait du bon travail. On va au parc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -2941,7 +3033,13 @@
       <c r="AV11" s="2" t="inlineStr"/>
       <c r="AW11" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|L'air du parc sent l'herbe coupée.
+narrateur|Nino a repris ses affaires.
+narrateur|C'était avant de partir.
+papa|Bravo, Nino.
+maman|Tu as fait du bon travail.
+enfant-m|On va au parc.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX11" t="inlineStr"/>
@@ -2969,7 +3067,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Maya s'arrête près de Léa. le ballon rouge est rangé. La lumière est claire. Maya souffle, puis sourit à maman. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>Nino a cherché la cuisine. Il a repris le ballon rouge. Maintenant, le manteau. Le cacao fume encore, tout petit. Nino prend le manteau. Il passe un bras, puis l'autre. Tout est près de la porte. Tu as repris tes affaires. C'est du bon travail. Mon manteau, maman. Nino reprend ses affaires, avant de partir. On a le seau. On a le manteau. On les prend. On peut sortir. Nino serre ce qu'il tient. Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -3109,7 +3207,19 @@
       <c r="AV12" s="2" t="inlineStr"/>
       <c r="AW12" t="inlineStr">
         <is>
-          <t>narrateur|Maya s'arrête près de Léa. le ballon rouge est rangé. La lumière est claire. Maya souffle, puis sourit à maman. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>narrateur|Nino a cherché la cuisine.
+narrateur|Il a repris le ballon rouge.
+narrateur|Maintenant, le manteau.
+narrateur|Le cacao fume encore, tout petit.
+narrateur|Nino prend le manteau. Il passe un bras, puis l'autre.
+narrateur|Tout est près de la porte.
+maman|Tu as repris tes affaires. C'est du bon travail.
+enfant-m|Mon manteau, maman.
+narrateur|Nino reprend ses affaires, avant de partir.
+maman|On a le seau. On a le manteau.
+papa|On les prend. On peut sortir.
+narrateur|Nino serre ce qu'il tient.
+enfant-m|Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="AX12" t="inlineStr"/>
@@ -3137,7 +3247,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Une flaque brille devant le portail. Nino a repris ses affaires. C'était avant de partir. Bravo, Nino. Tu as fait du bon travail. On va au parc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -3277,7 +3387,13 @@
       <c r="AV13" s="2" t="inlineStr"/>
       <c r="AW13" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Une flaque brille devant le portail.
+narrateur|Nino a repris ses affaires.
+narrateur|C'était avant de partir.
+papa|Bravo, Nino.
+maman|Tu as fait du bon travail.
+enfant-m|On va au parc.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX13" t="inlineStr"/>
@@ -3305,7 +3421,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Maya se souvient de la cuisine. Et de le ballon rouge. Et de Sami. Une cloche tinte, tout loin. Maya range la tasse. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>Nino a cherché la cuisine. Il a repris le ballon rouge. Maintenant, les chaussures. Un oiseau tape deux fois sur la gouttière. Nino enfile les chaussures. Elles font toc toc. Tout est près de la porte. On peut partir. Tu as repris ce qu'il fallait. Mes chaussures, papa. Nino reprend ses affaires, avant de partir. On a le seau. On a le manteau. On les prend. On peut sortir. Nino serre ce qu'il tient. Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -3445,7 +3561,19 @@
       <c r="AV14" s="2" t="inlineStr"/>
       <c r="AW14" t="inlineStr">
         <is>
-          <t>narrateur|Maya se souvient de la cuisine. Et de le ballon rouge. Et de Sami. Une cloche tinte, tout loin. Maya range la tasse. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>narrateur|Nino a cherché la cuisine.
+narrateur|Il a repris le ballon rouge.
+narrateur|Maintenant, les chaussures.
+narrateur|Un oiseau tape deux fois sur la gouttière.
+narrateur|Nino enfile les chaussures. Elles font toc toc.
+narrateur|Tout est près de la porte.
+papa|On peut partir. Tu as repris ce qu'il fallait.
+enfant-m|Mes chaussures, papa.
+narrateur|Nino reprend ses affaires, avant de partir.
+maman|On a le seau. On a le manteau.
+papa|On les prend. On peut sortir.
+narrateur|Nino serre ce qu'il tient.
+enfant-m|Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="AX14" t="inlineStr"/>
@@ -3473,7 +3601,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Le pain du matin sent encore, tout loin. Nino a repris ses affaires. C'était avant de partir. Bravo, Nino. Tu as fait du bon travail. On va au parc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -3613,7 +3741,13 @@
       <c r="AV15" s="2" t="inlineStr"/>
       <c r="AW15" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Le pain du matin sent encore, tout loin.
+narrateur|Nino a repris ses affaires.
+narrateur|C'était avant de partir.
+papa|Bravo, Nino.
+maman|Tu as fait du bon travail.
+enfant-m|On va au parc.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX15" t="inlineStr"/>
@@ -3641,7 +3775,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Maya trouve le seau bleu. Elle reprend ses affaires avant de partir. Elle le vide un peu. Encore le doudou. Je suis là. On va reprendre ses affaires avant de partir.</t>
+          <t>Nino est encore dans la cuisine. Ça sent encore le cacao. Le seau bleu est près de l'évier. Une goutte tombe dedans. Ploc. Le seau, Nino. Tu le reprends avant de partir ? Oui, papa. Le seau. Nino le soulève. Il est léger. Bravo. Tu le mets près de la porte. Le seau est sablé, léger. Nino pose le seau bleu près de la porte. Le carrelage est un peu froid. Nino tapote le bord du seau. Ça fait toc. Tu as repris le seau, avant de partir. Il vient au parc. On reprend ses affaires, avant de partir.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -3781,9 +3915,21 @@
       <c r="AV16" s="2" t="inlineStr"/>
       <c r="AW16" t="inlineStr">
         <is>
-          <t>narrateur|Maya trouve le seau bleu. Elle reprend ses affaires avant de partir. Elle le vide un peu.
-papa|Encore le doudou.
-maman|Je suis là. On va reprendre ses affaires avant de partir.</t>
+          <t>narrateur|Nino est encore dans la cuisine.
+narrateur|Ça sent encore le cacao.
+narrateur|Le seau bleu est près de l'évier.
+narrateur|Une goutte tombe dedans. Ploc.
+papa|Le seau, Nino. Tu le reprends avant de partir ?
+enfant-m|Oui, papa. Le seau.
+narrateur|Nino le soulève. Il est léger.
+maman|Bravo. Tu le mets près de la porte.
+narrateur|Le seau est sablé, léger.
+narrateur|Nino pose le seau bleu près de la porte.
+narrateur|Le carrelage est un peu froid.
+narrateur|Nino tapote le bord du seau. Ça fait toc.
+maman|Tu as repris le seau, avant de partir.
+enfant-m|Il vient au parc.
+maman|On reprend ses affaires, avant de partir.</t>
         </is>
       </c>
       <c r="AX16" t="inlineStr"/>
@@ -3811,7 +3957,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre Tom, Léa, ou Sami.</t>
+          <t>Il reste une chose, pour sortir. Le sac, le manteau, ou les chaussures ? Tu choisis, Nino.</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -3979,7 +4125,9 @@
       </c>
       <c r="AW17" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre Tom, Léa, ou Sami.</t>
+          <t>narrateur|Il reste une chose, pour sortir.
+papa|Le sac, le manteau, ou les chaussures ?
+maman|Tu choisis, Nino.</t>
         </is>
       </c>
       <c r="AX17" t="inlineStr"/>
@@ -4007,7 +4155,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Avec Tom. Après le seau bleu. Près de la cuisine. Maya s'arrête. On attend son tour. Maya prend la main de maman. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>Nino a cherché la cuisine. Il a repris le seau bleu. Maintenant, le sac. Le tapis garde un carré de soleil. Nino ouvre le sac. Il y glisse ce qu'il a repris. Tout est près de la porte. Avant de partir, tu as bien cherché. Bravo. C'est prêt. Nino reprend ses affaires, avant de partir. On a le seau. On a le manteau. On les prend. On peut sortir. Nino serre ce qu'il tient. Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -4147,10 +4295,26 @@
       <c r="AV18" s="2" t="inlineStr"/>
       <c r="AW18" t="inlineStr">
         <is>
-          <t>narrateur|Avec Tom. Après le seau bleu. Près de la cuisine. Maya s'arrête. On attend son tour. Maya prend la main de maman. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
-        </is>
-      </c>
-      <c r="AX18" t="inlineStr"/>
+          <t>narrateur|Nino a cherché la cuisine.
+narrateur|Il a repris le seau bleu.
+narrateur|Maintenant, le sac.
+narrateur|Le tapis garde un carré de soleil.
+narrateur|Nino ouvre le sac. Il y glisse ce qu'il a repris.
+narrateur|Tout est près de la porte.
+maman|Avant de partir, tu as bien cherché. Bravo.
+enfant-m|C'est prêt.
+narrateur|Nino reprend ses affaires, avant de partir.
+maman|On a le seau. On a le manteau.
+papa|On les prend. On peut sortir.
+narrateur|Nino serre ce qu'il tient.
+enfant-m|Merci, maman. Merci, papa.</t>
+        </is>
+      </c>
+      <c r="AX18" t="inlineStr">
+        <is>
+          <t>porte</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -4175,7 +4339,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Un vélo passe, tout doux. Nino a repris ses affaires. C'était avant de partir. Bravo, Nino. Tu as fait du bon travail. On va au parc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -4315,7 +4479,13 @@
       <c r="AV19" s="2" t="inlineStr"/>
       <c r="AW19" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Un vélo passe, tout doux.
+narrateur|Nino a repris ses affaires.
+narrateur|C'était avant de partir.
+papa|Bravo, Nino.
+maman|Tu as fait du bon travail.
+enfant-m|On va au parc.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX19" t="inlineStr"/>
@@ -4343,7 +4513,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Maya range le seau bleu. Léa reste près de la cuisine. Une pomme brille un peu. Maya écoute maman encore une fois. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>Nino a cherché la cuisine. Il a repris le seau bleu. Maintenant, le manteau. Les crochets de l'entrée font tic. Nino prend le manteau. Il passe un bras, puis l'autre. Tout est près de la porte. Le sac est prêt. Bravo, Nino. On peut partir ? Nino reprend ses affaires, avant de partir. On a le seau. On a le manteau. On les prend. On peut sortir. Nino serre ce qu'il tient. Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -4483,7 +4653,19 @@
       <c r="AV20" s="2" t="inlineStr"/>
       <c r="AW20" t="inlineStr">
         <is>
-          <t>narrateur|Maya range le seau bleu. Léa reste près de la cuisine. Une pomme brille un peu. Maya écoute maman encore une fois. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>narrateur|Nino a cherché la cuisine.
+narrateur|Il a repris le seau bleu.
+narrateur|Maintenant, le manteau.
+narrateur|Les crochets de l'entrée font tic.
+narrateur|Nino prend le manteau. Il passe un bras, puis l'autre.
+narrateur|Tout est près de la porte.
+papa|Le sac est prêt. Bravo, Nino.
+enfant-m|On peut partir ?
+narrateur|Nino reprend ses affaires, avant de partir.
+maman|On a le seau. On a le manteau.
+papa|On les prend. On peut sortir.
+narrateur|Nino serre ce qu'il tient.
+enfant-m|Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="AX20" t="inlineStr"/>
@@ -4511,7 +4693,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Le seau tape un peu la jambe de Nino. Nino a repris ses affaires. C'était avant de partir. Bravo, Nino. Tu as fait du bon travail. On va au parc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -4651,7 +4833,13 @@
       <c r="AV21" s="2" t="inlineStr"/>
       <c r="AW21" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Le seau tape un peu la jambe de Nino.
+narrateur|Nino a repris ses affaires.
+narrateur|C'était avant de partir.
+papa|Bravo, Nino.
+maman|Tu as fait du bon travail.
+enfant-m|On va au parc.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX21" t="inlineStr"/>
@@ -4679,7 +4867,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Sami est là. le seau bleu aussi. la cuisine reste dans le souvenir. Un panier est posé sur le banc. Papa n'est pas loin. Maya les rejoint. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>Nino a cherché la cuisine. Il a repris le seau bleu. Maintenant, les chaussures. Une cuillère tinte, loin, dans la cuisine. Nino enfile les chaussures. Elles font toc toc. Tout est près de la porte. Le manteau est bon. Tu as fait du bon travail. J'ai tout. Nino reprend ses affaires, avant de partir. On a le seau. On a le manteau. On les prend. On peut sortir. Nino serre ce qu'il tient. Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -4819,7 +5007,19 @@
       <c r="AV22" s="2" t="inlineStr"/>
       <c r="AW22" t="inlineStr">
         <is>
-          <t>narrateur|Sami est là. le seau bleu aussi. la cuisine reste dans le souvenir. Un panier est posé sur le banc. Papa n'est pas loin. Maya les rejoint. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>narrateur|Nino a cherché la cuisine.
+narrateur|Il a repris le seau bleu.
+narrateur|Maintenant, les chaussures.
+narrateur|Une cuillère tinte, loin, dans la cuisine.
+narrateur|Nino enfile les chaussures. Elles font toc toc.
+narrateur|Tout est près de la porte.
+maman|Le manteau est bon. Tu as fait du bon travail.
+enfant-m|J'ai tout.
+narrateur|Nino reprend ses affaires, avant de partir.
+maman|On a le seau. On a le manteau.
+papa|On les prend. On peut sortir.
+narrateur|Nino serre ce qu'il tient.
+enfant-m|Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="AX22" t="inlineStr"/>
@@ -4847,7 +5047,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Le manteau fait un bruit de tissu. Nino a repris ses affaires. C'était avant de partir. Bravo, Nino. Tu as fait du bon travail. On va au parc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -4987,7 +5187,13 @@
       <c r="AV23" s="2" t="inlineStr"/>
       <c r="AW23" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Le manteau fait un bruit de tissu.
+narrateur|Nino a repris ses affaires.
+narrateur|C'était avant de partir.
+papa|Bravo, Nino.
+maman|Tu as fait du bon travail.
+enfant-m|On va au parc.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX23" t="inlineStr"/>
@@ -5015,7 +5221,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Maya trouve le doudou. Elle reprend ses affaires avant de partir. Elle le serre. Encore le manteau. Maman reste tout près. On va reprendre ses affaires avant de partir.</t>
+          <t>Nino est encore dans la cuisine. Ça sent encore le cacao. Le doudou est sur une chaise. Il sent un peu le cacao. Ton doudou, Nino. Tu le reprends ? Oui. Mon doudou. Nino le serre contre sa joue. Bravo. Tu le mets près de la porte. Le doudou est chaud, un peu froissé. Nino serre le doudou, puis le pose près de la porte. Le carrelage est un peu froid. Nino remet l'oreille du doudou à sa place. Tu as repris le doudou, avant de partir. Il vient avec moi. On reprend ses affaires, avant de partir.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -5155,8 +5361,21 @@
       <c r="AV24" s="2" t="inlineStr"/>
       <c r="AW24" t="inlineStr">
         <is>
-          <t>narrateur|Maya trouve le doudou. Elle reprend ses affaires avant de partir. Elle le serre.
-maman|Encore le manteau. Maman reste tout près. On va reprendre ses affaires avant de partir.</t>
+          <t>narrateur|Nino est encore dans la cuisine.
+narrateur|Ça sent encore le cacao.
+narrateur|Le doudou est sur une chaise.
+narrateur|Il sent un peu le cacao.
+maman|Ton doudou, Nino. Tu le reprends ?
+enfant-m|Oui. Mon doudou.
+narrateur|Nino le serre contre sa joue.
+papa|Bravo. Tu le mets près de la porte.
+narrateur|Le doudou est chaud, un peu froissé.
+narrateur|Nino serre le doudou, puis le pose près de la porte.
+narrateur|Le carrelage est un peu froid.
+narrateur|Nino remet l'oreille du doudou à sa place.
+papa|Tu as repris le doudou, avant de partir.
+enfant-m|Il vient avec moi.
+maman|On reprend ses affaires, avant de partir.</t>
         </is>
       </c>
       <c r="AX24" t="inlineStr"/>
@@ -5184,7 +5403,7 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre Tom, Léa, ou Sami.</t>
+          <t>Il reste une chose, pour sortir. Le sac, le manteau, ou les chaussures ? Tu choisis, Nino.</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -5352,7 +5571,9 @@
       </c>
       <c r="AW25" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre Tom, Léa, ou Sami.</t>
+          <t>narrateur|Il reste une chose, pour sortir.
+papa|Le sac, le manteau, ou les chaussures ?
+maman|Tu choisis, Nino.</t>
         </is>
       </c>
       <c r="AX25" t="inlineStr"/>
@@ -5380,7 +5601,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Maya rejoint Tom. le doudou est rangé. la cuisine est fini. Ça sent le pain chaud. Maya raccroche un linge. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>Nino a cherché la cuisine. Il a repris le doudou. Maintenant, le sac. Le banc du jardin brille encore. Nino ouvre le sac. Il y glisse ce qu'il a repris. Tout est près de la porte. Les chaussures sont mises. Bravo. Le doudou vient. Nino reprend ses affaires, avant de partir. On a le seau. On a le manteau. On les prend. On peut sortir. Nino serre ce qu'il tient. Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -5520,10 +5741,26 @@
       <c r="AV26" s="2" t="inlineStr"/>
       <c r="AW26" t="inlineStr">
         <is>
-          <t>narrateur|Maya rejoint Tom. le doudou est rangé. la cuisine est fini. Ça sent le pain chaud. Maya raccroche un linge. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
-        </is>
-      </c>
-      <c r="AX26" t="inlineStr"/>
+          <t>narrateur|Nino a cherché la cuisine.
+narrateur|Il a repris le doudou.
+narrateur|Maintenant, le sac.
+narrateur|Le banc du jardin brille encore.
+narrateur|Nino ouvre le sac. Il y glisse ce qu'il a repris.
+narrateur|Tout est près de la porte.
+papa|Les chaussures sont mises. Bravo.
+enfant-m|Le doudou vient.
+narrateur|Nino reprend ses affaires, avant de partir.
+maman|On a le seau. On a le manteau.
+papa|On les prend. On peut sortir.
+narrateur|Nino serre ce qu'il tient.
+enfant-m|Merci, maman. Merci, papa.</t>
+        </is>
+      </c>
+      <c r="AX26" t="inlineStr">
+        <is>
+          <t>porte</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -5548,7 +5785,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Les chaussures font toc toc sur le gravier. Nino a repris ses affaires. C'était avant de partir. Bravo, Nino. Tu as fait du bon travail. On va au parc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -5688,7 +5925,13 @@
       <c r="AV27" s="2" t="inlineStr"/>
       <c r="AW27" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Les chaussures font toc toc sur le gravier.
+narrateur|Nino a repris ses affaires.
+narrateur|C'était avant de partir.
+papa|Bravo, Nino.
+maman|Tu as fait du bon travail.
+enfant-m|On va au parc.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX27" t="inlineStr"/>
@@ -5716,7 +5959,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Près de Léa. Maya pose le doudou. la cuisine est derrière. On se tient la main. Maya enfile ses chaussons. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>Nino a cherché la cuisine. Il a repris le doudou. Maintenant, le manteau. Une goutte tombe du rebord. Ploc. Nino prend le manteau. Il passe un bras, puis l'autre. Tout est près de la porte. Tu as repris le seau et le manteau. Bravo. Le seau est là. Nino reprend ses affaires, avant de partir. On a le seau. On a le manteau. On les prend. On peut sortir. Nino serre ce qu'il tient. Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -5856,7 +6099,19 @@
       <c r="AV28" s="2" t="inlineStr"/>
       <c r="AW28" t="inlineStr">
         <is>
-          <t>narrateur|Près de Léa. Maya pose le doudou. la cuisine est derrière. On se tient la main. Maya enfile ses chaussons. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>narrateur|Nino a cherché la cuisine.
+narrateur|Il a repris le doudou.
+narrateur|Maintenant, le manteau.
+narrateur|Une goutte tombe du rebord. Ploc.
+narrateur|Nino prend le manteau. Il passe un bras, puis l'autre.
+narrateur|Tout est près de la porte.
+maman|Tu as repris le seau et le manteau. Bravo.
+enfant-m|Le seau est là.
+narrateur|Nino reprend ses affaires, avant de partir.
+maman|On a le seau. On a le manteau.
+papa|On les prend. On peut sortir.
+narrateur|Nino serre ce qu'il tient.
+enfant-m|Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="AX28" t="inlineStr"/>
@@ -5884,7 +6139,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Le doudou regarde la rue, une oreille en l'air. Nino a repris ses affaires. C'était avant de partir. Bravo, Nino. Tu as fait du bon travail. On va au parc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -6024,7 +6279,13 @@
       <c r="AV29" s="2" t="inlineStr"/>
       <c r="AW29" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Le doudou regarde la rue, une oreille en l'air.
+narrateur|Nino a repris ses affaires.
+narrateur|C'était avant de partir.
+papa|Bravo, Nino.
+maman|Tu as fait du bon travail.
+enfant-m|On va au parc.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX29" t="inlineStr"/>
@@ -6052,7 +6313,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Maya montre Sami. Maman a vu la cuisine. Et le doudou. On entend un oiseau. Maya caresse le doudou. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>Nino a cherché la cuisine. Il a repris le doudou. Maintenant, les chaussures. Le rideau bouge un peu, tout seul. Nino enfile les chaussures. Elles font toc toc. Tout est près de la porte. On a tout, Nino. On peut ouvrir la porte. Le ballon aussi. Nino reprend ses affaires, avant de partir. On a le seau. On a le manteau. On les prend. On peut sortir. Nino serre ce qu'il tient. Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -6192,7 +6453,19 @@
       <c r="AV30" s="2" t="inlineStr"/>
       <c r="AW30" t="inlineStr">
         <is>
-          <t>narrateur|Maya montre Sami. Maman a vu la cuisine. Et le doudou. On entend un oiseau. Maya caresse le doudou. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>narrateur|Nino a cherché la cuisine.
+narrateur|Il a repris le doudou.
+narrateur|Maintenant, les chaussures.
+narrateur|Le rideau bouge un peu, tout seul.
+narrateur|Nino enfile les chaussures. Elles font toc toc.
+narrateur|Tout est près de la porte.
+papa|On a tout, Nino. On peut ouvrir la porte.
+enfant-m|Le ballon aussi.
+narrateur|Nino reprend ses affaires, avant de partir.
+maman|On a le seau. On a le manteau.
+papa|On les prend. On peut sortir.
+narrateur|Nino serre ce qu'il tient.
+enfant-m|Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="AX30" t="inlineStr"/>
@@ -6220,7 +6493,7 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Le ballon rouge rebondit une fois, contre la hanche. Nino a repris ses affaires. C'était avant de partir. Bravo, Nino. Tu as fait du bon travail. On va au parc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -6360,7 +6633,13 @@
       <c r="AV31" s="2" t="inlineStr"/>
       <c r="AW31" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Le ballon rouge rebondit une fois, contre la hanche.
+narrateur|Nino a repris ses affaires.
+narrateur|C'était avant de partir.
+papa|Bravo, Nino.
+maman|Tu as fait du bon travail.
+enfant-m|On va au parc.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX31" t="inlineStr"/>
@@ -6388,7 +6667,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Maya va dans le jardin. Elle cherche. Elle reprend ses affaires avant de partir. Un chapeau est sur le banc. Papa l'appelle. Maya le prend.</t>
+          <t>Nino ouvre la porte du jardin. L'air sent la terre mouillée. L'herbe brille encore. Un chapeau est sur le banc. Le chapeau est sur le banc, Nino. Tu le prends ? Oui, papa. Nino marche sur les dalles froides. Il prend le chapeau. Le ruban est un peu humide. Bravo. Tu reprends tes affaires. C'est avant de partir. Un oiseau crie une fois, tout près. On cherche aussi le seau et le manteau. Je cherche, papa.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -6528,7 +6807,21 @@
       <c r="AV32" s="2" t="inlineStr"/>
       <c r="AW32" t="inlineStr">
         <is>
-          <t>narrateur|Maya va dans le jardin. Elle cherche. Elle reprend ses affaires avant de partir. Un chapeau est sur le banc. Papa l'appelle. Maya le prend.</t>
+          <t>narrateur|Nino ouvre la porte du jardin.
+narrateur|L'air sent la terre mouillée.
+narrateur|L'herbe brille encore.
+narrateur|Un chapeau est sur le banc.
+papa|Le chapeau est sur le banc, Nino.
+papa|Tu le prends ?
+enfant-m|Oui, papa.
+narrateur|Nino marche sur les dalles froides.
+narrateur|Il prend le chapeau.
+narrateur|Le ruban est un peu humide.
+maman|Bravo. Tu reprends tes affaires.
+maman|C'est avant de partir.
+narrateur|Un oiseau crie une fois, tout près.
+papa|On cherche aussi le seau et le manteau.
+enfant-m|Je cherche, papa.</t>
         </is>
       </c>
       <c r="AX32" t="inlineStr"/>
@@ -6744,7 +7037,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Oui. On va reprendre ses affaires avant de partir. Maya retient le geste. Maman sourit. On va reprendre ses affaires avant de partir.</t>
+          <t>Oui. Nino a repris le chapeau. Il le met près de lui. Bravo, Nino. Tu as fait du bon travail. Avant de partir, on reprend ses affaires. Le chapeau est là. Nino essuie ses mains sur son pantalon. Il regarde encore le jardin.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -6888,7 +7181,14 @@
       </c>
       <c r="AW34" t="inlineStr">
         <is>
-          <t>narrateur|Oui. On va reprendre ses affaires avant de partir. Maya retient le geste. Maman sourit. On va reprendre ses affaires avant de partir.</t>
+          <t>narrateur|Oui.
+narrateur|Nino a repris le chapeau.
+narrateur|Il le met près de lui.
+papa|Bravo, Nino. Tu as fait du bon travail.
+maman|Avant de partir, on reprend ses affaires.
+enfant-m|Le chapeau est là.
+narrateur|Nino essuie ses mains sur son pantalon.
+narrateur|Il regarde encore le jardin.</t>
         </is>
       </c>
       <c r="AX34" t="inlineStr"/>
@@ -6916,7 +7216,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre le ballon rouge, le seau bleu, ou le doudou.</t>
+          <t>Quel objet Nino reprend, dans le jardin ? Le ballon rouge, le seau bleu, ou le doudou ?</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -7080,7 +7380,8 @@
       <c r="AV35" s="2" t="inlineStr"/>
       <c r="AW35" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre le ballon rouge, le seau bleu, ou le doudou.</t>
+          <t>narrateur|Quel objet Nino reprend, dans le jardin ?
+papa|Le ballon rouge, le seau bleu, ou le doudou ?</t>
         </is>
       </c>
       <c r="AX35" t="inlineStr"/>
@@ -7108,7 +7409,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Maya retrouve Tom. Tom tient le ballon. Maya reprend ses affaires avant de partir. J'ai le ballon. Je suis là. On va reprendre ses affaires avant de partir.</t>
+          <t>Nino est encore dans le jardin. L'air sent la terre mouillée. Le ballon rouge est dans l'herbe. Il est un peu mouillé, tout brillant. Le ballon, Nino. Tu le reprends ? Oui. Il est froid ! Nino le prend à deux mains. Bravo. Tu le mets près de la porte. Le ballon est lisse, un peu poussiéreux. Nino pose le ballon rouge près de la porte. L'herbe colle un peu aux chaussons. Nino souffle sur le ballon. Un peu de poussière part. Tu as repris le ballon, avant de partir. Il vient au parc. On reprend ses affaires, avant de partir.</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -7248,9 +7549,21 @@
       <c r="AV36" s="2" t="inlineStr"/>
       <c r="AW36" t="inlineStr">
         <is>
-          <t>narrateur|Maya retrouve Tom. Tom tient le ballon. Maya reprend ses affaires avant de partir.
-narrateur|J'ai le ballon.
-maman|Je suis là. On va reprendre ses affaires avant de partir.</t>
+          <t>narrateur|Nino est encore dans le jardin.
+narrateur|L'air sent la terre mouillée.
+narrateur|Le ballon rouge est dans l'herbe.
+narrateur|Il est un peu mouillé, tout brillant.
+papa|Le ballon, Nino. Tu le reprends ?
+enfant-m|Oui. Il est froid !
+narrateur|Nino le prend à deux mains.
+maman|Bravo. Tu le mets près de la porte.
+narrateur|Le ballon est lisse, un peu poussiéreux.
+narrateur|Nino pose le ballon rouge près de la porte.
+narrateur|L'herbe colle un peu aux chaussons.
+narrateur|Nino souffle sur le ballon. Un peu de poussière part.
+papa|Tu as repris le ballon, avant de partir.
+enfant-m|Il vient au parc.
+maman|On reprend ses affaires, avant de partir.</t>
         </is>
       </c>
       <c r="AX36" t="inlineStr"/>
@@ -7278,7 +7591,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre Tom, Léa, ou Sami.</t>
+          <t>Il reste une chose, pour sortir. Le sac, le manteau, ou les chaussures ? Tu choisis, Nino.</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -7446,7 +7759,9 @@
       </c>
       <c r="AW37" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre Tom, Léa, ou Sami.</t>
+          <t>narrateur|Il reste une chose, pour sortir.
+papa|Le sac, le manteau, ou les chaussures ?
+maman|Tu choisis, Nino.</t>
         </is>
       </c>
       <c r="AX37" t="inlineStr"/>
@@ -7474,7 +7789,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Maya a choisi le jardin. Puis le ballon rouge. Puis Tom. Un ruban reste dans la poche. Maya répète tout bas le geste. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>Nino a cherché le jardin. Il a repris le ballon rouge. Maintenant, le sac. Le savon de la chambre sent encore. Nino ouvre le sac. Il y glisse ce qu'il a repris. Tout est près de la porte. Merci, Nino. Tu as repris tes affaires. Merci, papa. Nino reprend ses affaires, avant de partir. On a le seau. On a le manteau. On les prend. On peut sortir. Nino serre ce qu'il tient. Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -7614,10 +7929,26 @@
       <c r="AV38" s="2" t="inlineStr"/>
       <c r="AW38" t="inlineStr">
         <is>
-          <t>narrateur|Maya a choisi le jardin. Puis le ballon rouge. Puis Tom. Un ruban reste dans la poche. Maya répète tout bas le geste. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
-        </is>
-      </c>
-      <c r="AX38" t="inlineStr"/>
+          <t>narrateur|Nino a cherché le jardin.
+narrateur|Il a repris le ballon rouge.
+narrateur|Maintenant, le sac.
+narrateur|Le savon de la chambre sent encore.
+narrateur|Nino ouvre le sac. Il y glisse ce qu'il a repris.
+narrateur|Tout est près de la porte.
+maman|Merci, Nino. Tu as repris tes affaires.
+enfant-m|Merci, papa.
+narrateur|Nino reprend ses affaires, avant de partir.
+maman|On a le seau. On a le manteau.
+papa|On les prend. On peut sortir.
+narrateur|Nino serre ce qu'il tient.
+enfant-m|Merci, maman. Merci, papa.</t>
+        </is>
+      </c>
+      <c r="AX38" t="inlineStr">
+        <is>
+          <t>porte</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -7642,7 +7973,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Le sac est un peu lourd, bien fermé. Nino a repris ses affaires. C'était avant de partir. Bravo, Nino. Tu as fait du bon travail. On va au parc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -7782,7 +8113,13 @@
       <c r="AV39" s="2" t="inlineStr"/>
       <c r="AW39" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Le sac est un peu lourd, bien fermé.
+narrateur|Nino a repris ses affaires.
+narrateur|C'était avant de partir.
+papa|Bravo, Nino.
+maman|Tu as fait du bon travail.
+enfant-m|On va au parc.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX39" t="inlineStr"/>
@@ -7810,7 +8147,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Maya s'arrête près de Léa. le ballon rouge est rangé. Il y a des miettes sur la table. Maya chuchote : c'est fini. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>Nino a cherché le jardin. Il a repris le ballon rouge. Maintenant, le manteau. Un galet froid attend sur le paillasson. Nino prend le manteau. Il passe un bras, puis l'autre. Tout est près de la porte. Tu as fini de ranger près de la porte ? Merci, maman. Nino reprend ses affaires, avant de partir. On a le seau. On a le manteau. On les prend. On peut sortir. Nino serre ce qu'il tient. Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -7950,7 +8287,19 @@
       <c r="AV40" s="2" t="inlineStr"/>
       <c r="AW40" t="inlineStr">
         <is>
-          <t>narrateur|Maya s'arrête près de Léa. le ballon rouge est rangé. Il y a des miettes sur la table. Maya chuchote : c'est fini. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>narrateur|Nino a cherché le jardin.
+narrateur|Il a repris le ballon rouge.
+narrateur|Maintenant, le manteau.
+narrateur|Un galet froid attend sur le paillasson.
+narrateur|Nino prend le manteau. Il passe un bras, puis l'autre.
+narrateur|Tout est près de la porte.
+papa|Tu as fini de ranger près de la porte ?
+enfant-m|Merci, maman.
+narrateur|Nino reprend ses affaires, avant de partir.
+maman|On a le seau. On a le manteau.
+papa|On les prend. On peut sortir.
+narrateur|Nino serre ce qu'il tient.
+enfant-m|Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="AX40" t="inlineStr"/>
@@ -7978,7 +8327,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Un chat traverse le muret, sans bruit. Nino a repris ses affaires. C'était avant de partir. Bravo, Nino. Tu as fait du bon travail. On va au parc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -8118,7 +8467,13 @@
       <c r="AV41" s="2" t="inlineStr"/>
       <c r="AW41" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Un chat traverse le muret, sans bruit.
+narrateur|Nino a repris ses affaires.
+narrateur|C'était avant de partir.
+papa|Bravo, Nino.
+maman|Tu as fait du bon travail.
+enfant-m|On va au parc.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX41" t="inlineStr"/>
@@ -8146,7 +8501,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Maya se souvient de le jardin. Et de le ballon rouge. Et de Sami. On écoute jusqu'au bout. Maya ferme le sac. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>Nino a cherché le jardin. Il a repris le ballon rouge. Maintenant, les chaussures. La chaise de l'entrée ne bouge plus. Nino enfile les chaussures. Elles font toc toc. Tout est près de la porte. Tu as le doudou ? Très bien. Je tiens le sac. Nino reprend ses affaires, avant de partir. On a le seau. On a le manteau. On les prend. On peut sortir. Nino serre ce qu'il tient. Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -8286,7 +8641,19 @@
       <c r="AV42" s="2" t="inlineStr"/>
       <c r="AW42" t="inlineStr">
         <is>
-          <t>narrateur|Maya se souvient de le jardin. Et de le ballon rouge. Et de Sami. On écoute jusqu'au bout. Maya ferme le sac. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>narrateur|Nino a cherché le jardin.
+narrateur|Il a repris le ballon rouge.
+narrateur|Maintenant, les chaussures.
+narrateur|La chaise de l'entrée ne bouge plus.
+narrateur|Nino enfile les chaussures. Elles font toc toc.
+narrateur|Tout est près de la porte.
+maman|Tu as le doudou ? Très bien.
+enfant-m|Je tiens le sac.
+narrateur|Nino reprend ses affaires, avant de partir.
+maman|On a le seau. On a le manteau.
+papa|On les prend. On peut sortir.
+narrateur|Nino serre ce qu'il tient.
+enfant-m|Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="AX42" t="inlineStr"/>
@@ -8314,7 +8681,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>La gouttière goutte encore, tout petit. Nino a repris ses affaires. C'était avant de partir. Bravo, Nino. Tu as fait du bon travail. On va au parc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -8454,7 +8821,13 @@
       <c r="AV43" s="2" t="inlineStr"/>
       <c r="AW43" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|La gouttière goutte encore, tout petit.
+narrateur|Nino a repris ses affaires.
+narrateur|C'était avant de partir.
+papa|Bravo, Nino.
+maman|Tu as fait du bon travail.
+enfant-m|On va au parc.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX43" t="inlineStr"/>
@@ -8482,7 +8855,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Maya retrouve Léa. Léa tient le seau. Maya reprend ses affaires avant de partir. J'ai le seau. Maman reste tout près. On va reprendre ses affaires avant de partir.</t>
+          <t>Nino est encore dans le jardin. L'air sent la terre mouillée. Le seau bleu est près du romarin. Une feuille est tombée dedans. Le seau, Nino. Tu le vides un peu ? Je le prends, maman. Nino verse la feuille sur la terre. Bravo. Tu le mets près de la porte. Le seau est sablé, léger. Nino pose le seau bleu près de la porte. L'herbe colle un peu aux chaussons. Nino tapote le bord du seau. Ça fait toc. Tu as repris le seau, avant de partir. Il vient au parc. On reprend ses affaires, avant de partir.</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -8622,8 +8995,21 @@
       <c r="AV44" s="2" t="inlineStr"/>
       <c r="AW44" t="inlineStr">
         <is>
-          <t>narrateur|Maya retrouve Léa. Léa tient le seau. Maya reprend ses affaires avant de partir.
-narrateur|J'ai le seau. Maman reste tout près. On va reprendre ses affaires avant de partir.</t>
+          <t>narrateur|Nino est encore dans le jardin.
+narrateur|L'air sent la terre mouillée.
+narrateur|Le seau bleu est près du romarin.
+narrateur|Une feuille est tombée dedans.
+maman|Le seau, Nino. Tu le vides un peu ?
+enfant-m|Je le prends, maman.
+narrateur|Nino verse la feuille sur la terre.
+papa|Bravo. Tu le mets près de la porte.
+narrateur|Le seau est sablé, léger.
+narrateur|Nino pose le seau bleu près de la porte.
+narrateur|L'herbe colle un peu aux chaussons.
+narrateur|Nino tapote le bord du seau. Ça fait toc.
+maman|Tu as repris le seau, avant de partir.
+enfant-m|Il vient au parc.
+maman|On reprend ses affaires, avant de partir.</t>
         </is>
       </c>
       <c r="AX44" t="inlineStr"/>
@@ -8651,7 +9037,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre Tom, Léa, ou Sami.</t>
+          <t>Il reste une chose, pour sortir. Le sac, le manteau, ou les chaussures ? Tu choisis, Nino.</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -8819,7 +9205,9 @@
       </c>
       <c r="AW45" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre Tom, Léa, ou Sami.</t>
+          <t>narrateur|Il reste une chose, pour sortir.
+papa|Le sac, le manteau, ou les chaussures ?
+maman|Tu choisis, Nino.</t>
         </is>
       </c>
       <c r="AX45" t="inlineStr"/>
@@ -8847,7 +9235,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Avec Tom. Après le seau bleu. Près de le jardin. Maya s'arrête. On dit merci. J'ai appris. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>Nino a cherché le jardin. Il a repris le seau bleu. Maintenant, le sac. Le sac a un zip qui chante. Nino ouvre le sac. Il y glisse ce qu'il a repris. Tout est près de la porte. On y va. Tes affaires sont avec toi. Le manteau est chaud. Nino reprend ses affaires, avant de partir. On a le seau. On a le manteau. On les prend. On peut sortir. Nino serre ce qu'il tient. Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -8987,12 +9375,26 @@
       <c r="AV46" s="2" t="inlineStr"/>
       <c r="AW46" t="inlineStr">
         <is>
-          <t>narrateur|Avec Tom. Après le seau bleu. Près de le jardin. Maya s'arrête. On dit merci.
-enfant-f|J'ai appris. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires.
-narrateur|Maya dit merci à maman.</t>
-        </is>
-      </c>
-      <c r="AX46" t="inlineStr"/>
+          <t>narrateur|Nino a cherché le jardin.
+narrateur|Il a repris le seau bleu.
+narrateur|Maintenant, le sac.
+narrateur|Le sac a un zip qui chante.
+narrateur|Nino ouvre le sac. Il y glisse ce qu'il a repris.
+narrateur|Tout est près de la porte.
+papa|On y va. Tes affaires sont avec toi.
+enfant-m|Le manteau est chaud.
+narrateur|Nino reprend ses affaires, avant de partir.
+maman|On a le seau. On a le manteau.
+papa|On les prend. On peut sortir.
+narrateur|Nino serre ce qu'il tient.
+enfant-m|Merci, maman. Merci, papa.</t>
+        </is>
+      </c>
+      <c r="AX46" t="inlineStr">
+        <is>
+          <t>porte</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -9017,7 +9419,7 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Le soleil a séché le banc du jardin. Nino a repris ses affaires. C'était avant de partir. Bravo, Nino. Tu as fait du bon travail. On va au parc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -9157,7 +9559,13 @@
       <c r="AV47" s="2" t="inlineStr"/>
       <c r="AW47" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Le soleil a séché le banc du jardin.
+narrateur|Nino a repris ses affaires.
+narrateur|C'était avant de partir.
+papa|Bravo, Nino.
+maman|Tu as fait du bon travail.
+enfant-m|On va au parc.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX47" t="inlineStr"/>
@@ -9185,7 +9593,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Maya range le seau bleu. Léa reste près de le jardin. On souffle doucement. Maya montre Léa à maman. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>Nino a cherché le jardin. Il a repris le seau bleu. Maintenant, le manteau. Le manteau sent le vent d'hier. Nino prend le manteau. Il passe un bras, puis l'autre. Tout est près de la porte. Bravo. C'est calme, maintenant. Toc toc, mes chaussures. Nino reprend ses affaires, avant de partir. On a le seau. On a le manteau. On les prend. On peut sortir. Nino serre ce qu'il tient. Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -9325,7 +9733,19 @@
       <c r="AV48" s="2" t="inlineStr"/>
       <c r="AW48" t="inlineStr">
         <is>
-          <t>narrateur|Maya range le seau bleu. Léa reste près de le jardin. On souffle doucement. Maya montre Léa à maman. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>narrateur|Nino a cherché le jardin.
+narrateur|Il a repris le seau bleu.
+narrateur|Maintenant, le manteau.
+narrateur|Le manteau sent le vent d'hier.
+narrateur|Nino prend le manteau. Il passe un bras, puis l'autre.
+narrateur|Tout est près de la porte.
+maman|Bravo. C'est calme, maintenant.
+enfant-m|Toc toc, mes chaussures.
+narrateur|Nino reprend ses affaires, avant de partir.
+maman|On a le seau. On a le manteau.
+papa|On les prend. On peut sortir.
+narrateur|Nino serre ce qu'il tient.
+enfant-m|Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="AX48" t="inlineStr"/>
@@ -9353,7 +9773,7 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Nino sent le cacao sur ses mains. Nino a repris ses affaires. C'était avant de partir. Bravo, Nino. Tu as fait du bon travail. On va au parc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -9493,7 +9913,13 @@
       <c r="AV49" s="2" t="inlineStr"/>
       <c r="AW49" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Nino sent le cacao sur ses mains.
+narrateur|Nino a repris ses affaires.
+narrateur|C'était avant de partir.
+papa|Bravo, Nino.
+maman|Tu as fait du bon travail.
+enfant-m|On va au parc.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX49" t="inlineStr"/>
@@ -9521,7 +9947,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Sami est là. le seau bleu aussi. le jardin reste dans le souvenir. On range un objet. Maya essuie ses mains. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>Nino a cherché le jardin. Il a repris le seau bleu. Maintenant, les chaussures. Les chaussures sont un peu sablées. Nino enfile les chaussures. Elles font toc toc. Tout est près de la porte. Tu as repris le ballon. Il vient avec nous. On va au parc. Nino reprend ses affaires, avant de partir. On a le seau. On a le manteau. On les prend. On peut sortir. Nino serre ce qu'il tient. Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -9661,7 +10087,19 @@
       <c r="AV50" s="2" t="inlineStr"/>
       <c r="AW50" t="inlineStr">
         <is>
-          <t>narrateur|Sami est là. le seau bleu aussi. le jardin reste dans le souvenir. On range un objet. Maya essuie ses mains. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>narrateur|Nino a cherché le jardin.
+narrateur|Il a repris le seau bleu.
+narrateur|Maintenant, les chaussures.
+narrateur|Les chaussures sont un peu sablées.
+narrateur|Nino enfile les chaussures. Elles font toc toc.
+narrateur|Tout est près de la porte.
+papa|Tu as repris le ballon. Il vient avec nous.
+enfant-m|On va au parc.
+narrateur|Nino reprend ses affaires, avant de partir.
+maman|On a le seau. On a le manteau.
+papa|On les prend. On peut sortir.
+narrateur|Nino serre ce qu'il tient.
+enfant-m|Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="AX50" t="inlineStr"/>
@@ -9689,7 +10127,7 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Le portail grince, puis s'ouvre. Nino a repris ses affaires. C'était avant de partir. Bravo, Nino. Tu as fait du bon travail. On va au parc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -9829,7 +10267,13 @@
       <c r="AV51" s="2" t="inlineStr"/>
       <c r="AW51" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Le portail grince, puis s'ouvre.
+narrateur|Nino a repris ses affaires.
+narrateur|C'était avant de partir.
+papa|Bravo, Nino.
+maman|Tu as fait du bon travail.
+enfant-m|On va au parc.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX51" t="inlineStr"/>
@@ -9857,7 +10301,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Maya retrouve Sami. Sami tient le doudou. Maya reprend ses affaires avant de partir. J'ai le doudou. Maman montre le geste, lentement. On va reprendre ses affaires avant de partir.</t>
+          <t>Nino est encore dans le jardin. L'air sent la terre mouillée. Le doudou est sur le banc, près du chapeau. Il a une goutte sur l'oreille. Ton doudou, Nino. Tu le reprends ? Oui, papa. Nino l'essuie sur son pull. Bravo. Tu le mets près de la porte. Le doudou est chaud, un peu froissé. Nino serre le doudou, puis le pose près de la porte. L'herbe colle un peu aux chaussons. Nino remet l'oreille du doudou à sa place. Tu as repris le doudou, avant de partir. Il vient avec moi. On reprend ses affaires, avant de partir.</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -9997,8 +10441,21 @@
       <c r="AV52" s="2" t="inlineStr"/>
       <c r="AW52" t="inlineStr">
         <is>
-          <t>narrateur|Maya retrouve Sami. Sami tient le doudou. Maya reprend ses affaires avant de partir.
-narrateur|J'ai le doudou. Maman montre le geste, lentement. On va reprendre ses affaires avant de partir.</t>
+          <t>narrateur|Nino est encore dans le jardin.
+narrateur|L'air sent la terre mouillée.
+narrateur|Le doudou est sur le banc, près du chapeau.
+narrateur|Il a une goutte sur l'oreille.
+papa|Ton doudou, Nino. Tu le reprends ?
+enfant-m|Oui, papa.
+narrateur|Nino l'essuie sur son pull.
+maman|Bravo. Tu le mets près de la porte.
+narrateur|Le doudou est chaud, un peu froissé.
+narrateur|Nino serre le doudou, puis le pose près de la porte.
+narrateur|L'herbe colle un peu aux chaussons.
+narrateur|Nino remet l'oreille du doudou à sa place.
+papa|Tu as repris le doudou, avant de partir.
+enfant-m|Il vient avec moi.
+maman|On reprend ses affaires, avant de partir.</t>
         </is>
       </c>
       <c r="AX52" t="inlineStr"/>
@@ -10026,7 +10483,7 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre Tom, Léa, ou Sami.</t>
+          <t>Il reste une chose, pour sortir. Le sac, le manteau, ou les chaussures ? Tu choisis, Nino.</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -10194,7 +10651,9 @@
       </c>
       <c r="AW53" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre Tom, Léa, ou Sami.</t>
+          <t>narrateur|Il reste une chose, pour sortir.
+papa|Le sac, le manteau, ou les chaussures ?
+maman|Tu choisis, Nino.</t>
         </is>
       </c>
       <c r="AX53" t="inlineStr"/>
@@ -10222,7 +10681,7 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Maya rejoint Tom. le doudou est rangé. le jardin est fini. Un chat miaule une fois. Maya dit merci à maman. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>Nino a cherché le jardin. Il a repris le doudou. Maintenant, le sac. Un rayon touche le seau bleu. Nino ouvre le sac. Il y glisse ce qu'il a repris. Tout est près de la porte. Avant de partir, on a tout repris. J'ai repris mes affaires. Nino reprend ses affaires, avant de partir. On a le seau. On a le manteau. On les prend. On peut sortir. Nino serre ce qu'il tient. Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -10362,10 +10821,26 @@
       <c r="AV54" s="2" t="inlineStr"/>
       <c r="AW54" t="inlineStr">
         <is>
-          <t>narrateur|Maya rejoint Tom. le doudou est rangé. le jardin est fini. Un chat miaule une fois. Maya dit merci à maman. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
-        </is>
-      </c>
-      <c r="AX54" t="inlineStr"/>
+          <t>narrateur|Nino a cherché le jardin.
+narrateur|Il a repris le doudou.
+narrateur|Maintenant, le sac.
+narrateur|Un rayon touche le seau bleu.
+narrateur|Nino ouvre le sac. Il y glisse ce qu'il a repris.
+narrateur|Tout est près de la porte.
+maman|Avant de partir, on a tout repris.
+enfant-m|J'ai repris mes affaires.
+narrateur|Nino reprend ses affaires, avant de partir.
+maman|On a le seau. On a le manteau.
+papa|On les prend. On peut sortir.
+narrateur|Nino serre ce qu'il tient.
+enfant-m|Merci, maman. Merci, papa.</t>
+        </is>
+      </c>
+      <c r="AX54" t="inlineStr">
+        <is>
+          <t>porte</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -10390,7 +10865,7 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Une feuille tourne sur le trottoir. Nino a repris ses affaires. C'était avant de partir. Bravo, Nino. Tu as fait du bon travail. On va au parc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -10530,7 +11005,13 @@
       <c r="AV55" s="2" t="inlineStr"/>
       <c r="AW55" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Une feuille tourne sur le trottoir.
+narrateur|Nino a repris ses affaires.
+narrateur|C'était avant de partir.
+papa|Bravo, Nino.
+maman|Tu as fait du bon travail.
+enfant-m|On va au parc.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX55" t="inlineStr"/>
@@ -10558,7 +11039,7 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Près de Léa. Maya pose le doudou. le jardin est derrière. La couverture est douce. Maya tend Léa à papa. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>Nino a cherché le jardin. Il a repris le doudou. Maintenant, le manteau. Le ballon rouge fait une ombre ronde. Nino prend le manteau. Il passe un bras, puis l'autre. Tout est près de la porte. Nino, tu as fait du bon travail. C'est lourd un peu. Nino reprend ses affaires, avant de partir. On a le seau. On a le manteau. On les prend. On peut sortir. Nino serre ce qu'il tient. Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -10698,7 +11179,19 @@
       <c r="AV56" s="2" t="inlineStr"/>
       <c r="AW56" t="inlineStr">
         <is>
-          <t>narrateur|Près de Léa. Maya pose le doudou. le jardin est derrière. La couverture est douce. Maya tend Léa à papa. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>narrateur|Nino a cherché le jardin.
+narrateur|Il a repris le doudou.
+narrateur|Maintenant, le manteau.
+narrateur|Le ballon rouge fait une ombre ronde.
+narrateur|Nino prend le manteau. Il passe un bras, puis l'autre.
+narrateur|Tout est près de la porte.
+papa|Nino, tu as fait du bon travail.
+enfant-m|C'est lourd un peu.
+narrateur|Nino reprend ses affaires, avant de partir.
+maman|On a le seau. On a le manteau.
+papa|On les prend. On peut sortir.
+narrateur|Nino serre ce qu'il tient.
+enfant-m|Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="AX56" t="inlineStr"/>
@@ -10726,7 +11219,7 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Le parc n'est pas loin. On entend un oiseau. Nino a repris ses affaires. C'était avant de partir. Bravo, Nino. Tu as fait du bon travail. On va au parc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -10866,7 +11359,13 @@
       <c r="AV57" s="2" t="inlineStr"/>
       <c r="AW57" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Le parc n'est pas loin. On entend un oiseau.
+narrateur|Nino a repris ses affaires.
+narrateur|C'était avant de partir.
+papa|Bravo, Nino.
+maman|Tu as fait du bon travail.
+enfant-m|On va au parc.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX57" t="inlineStr"/>
@@ -10894,7 +11393,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Maya montre Sami. Maman a vu le jardin. Et le doudou. Un crochet tient bien le manteau. Maya plie un pull. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>Nino a cherché le jardin. Il a repris le doudou. Maintenant, les chaussures. Le doudou a une oreille pliée. Nino enfile les chaussures. Elles font toc toc. Tout est près de la porte. On sort ensemble. Tes affaires sont prêtes. Je suis prêt. Nino reprend ses affaires, avant de partir. On a le seau. On a le manteau. On les prend. On peut sortir. Nino serre ce qu'il tient. Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -11034,7 +11533,19 @@
       <c r="AV58" s="2" t="inlineStr"/>
       <c r="AW58" t="inlineStr">
         <is>
-          <t>narrateur|Maya montre Sami. Maman a vu le jardin. Et le doudou. Un crochet tient bien le manteau. Maya plie un pull. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>narrateur|Nino a cherché le jardin.
+narrateur|Il a repris le doudou.
+narrateur|Maintenant, les chaussures.
+narrateur|Le doudou a une oreille pliée.
+narrateur|Nino enfile les chaussures. Elles font toc toc.
+narrateur|Tout est près de la porte.
+maman|On sort ensemble. Tes affaires sont prêtes.
+enfant-m|Je suis prêt.
+narrateur|Nino reprend ses affaires, avant de partir.
+maman|On a le seau. On a le manteau.
+papa|On les prend. On peut sortir.
+narrateur|Nino serre ce qu'il tient.
+enfant-m|Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="AX58" t="inlineStr"/>
@@ -11062,7 +11573,7 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Nino serre la main de maman. Nino a repris ses affaires. C'était avant de partir. Bravo, Nino. Tu as fait du bon travail. On va au parc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
@@ -11202,7 +11713,13 @@
       <c r="AV59" s="2" t="inlineStr"/>
       <c r="AW59" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Nino serre la main de maman.
+narrateur|Nino a repris ses affaires.
+narrateur|C'était avant de partir.
+papa|Bravo, Nino.
+maman|Tu as fait du bon travail.
+enfant-m|On va au parc.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX59" t="inlineStr"/>
@@ -11230,7 +11747,7 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Maya va dans la chambre. Elle cherche. Elle reprend ses affaires avant de partir. Un chausson est sous le lit. On les reprend. Maya le glisse dans le sac.</t>
+          <t>Nino va dans la chambre. Le rideau est encore un peu fermé. La couverture est douce, froissée. Un chausson est sous le lit. Regarde sous le lit, Nino. J'ai le chausson ! Nino le glisse près de l'autre. Les deux chaussons se touchent. Bravo. Tu reprends tes affaires, avant de partir. La chambre sent le savon, tout doux. On cherche aussi le seau et le manteau. Je continue, maman.</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -11370,9 +11887,18 @@
       <c r="AV60" s="2" t="inlineStr"/>
       <c r="AW60" t="inlineStr">
         <is>
-          <t>narrateur|Maya va dans la chambre. Elle cherche. Elle reprend ses affaires avant de partir. Un chausson est sous le lit.
-maman|On les reprend.
-narrateur|Maya le glisse dans le sac.</t>
+          <t>narrateur|Nino va dans la chambre.
+narrateur|Le rideau est encore un peu fermé.
+narrateur|La couverture est douce, froissée.
+narrateur|Un chausson est sous le lit.
+maman|Regarde sous le lit, Nino.
+enfant-m|J'ai le chausson !
+narrateur|Nino le glisse près de l'autre.
+narrateur|Les deux chaussons se touchent.
+papa|Bravo. Tu reprends tes affaires, avant de partir.
+narrateur|La chambre sent le savon, tout doux.
+maman|On cherche aussi le seau et le manteau.
+enfant-m|Je continue, maman.</t>
         </is>
       </c>
       <c r="AX60" t="inlineStr"/>
@@ -11588,7 +12114,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Oui. On va reprendre ses affaires avant de partir. Maya hoche la tête. On continue, avec maman. On va reprendre ses affaires avant de partir.</t>
+          <t>Oui. Nino a repris le chausson. La paire est complète. Bravo, Nino. C'est du bon travail. Avant de partir, on reprend ses affaires. C'est prêt, presque. Nino pose la main sur la couverture. Il est calme.</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -11732,7 +12258,14 @@
       </c>
       <c r="AW62" t="inlineStr">
         <is>
-          <t>narrateur|Oui. On va reprendre ses affaires avant de partir. Maya hoche la tête. On continue, avec maman. On va reprendre ses affaires avant de partir.</t>
+          <t>narrateur|Oui.
+narrateur|Nino a repris le chausson.
+narrateur|La paire est complète.
+maman|Bravo, Nino. C'est du bon travail.
+papa|Avant de partir, on reprend ses affaires.
+enfant-m|C'est prêt, presque.
+narrateur|Nino pose la main sur la couverture.
+narrateur|Il est calme.</t>
         </is>
       </c>
       <c r="AX62" t="inlineStr"/>
@@ -11760,7 +12293,7 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre le ballon rouge, le seau bleu, ou le doudou.</t>
+          <t>Quel objet Nino reprend, dans la chambre ? Le ballon rouge, le seau bleu, ou le doudou ?</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -11924,7 +12457,8 @@
       <c r="AV63" s="2" t="inlineStr"/>
       <c r="AW63" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre le ballon rouge, le seau bleu, ou le doudou.</t>
+          <t>narrateur|Quel objet Nino reprend, dans la chambre ?
+maman|Le ballon rouge, le seau bleu, ou le doudou ?</t>
         </is>
       </c>
       <c r="AX63" t="inlineStr"/>
@@ -11952,7 +12486,7 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Maya range le ballon, puis cherche encore. Elle reprend ses affaires avant de partir. Un gant manque. Elle le trouve. Maman reste tout près. On va reprendre ses affaires avant de partir.</t>
+          <t>Nino est encore dans la chambre. La chambre sent le savon doux. Le ballon rouge est sous le lit. Il touche le deuxième chausson. Le ballon, Nino. Tu le reprends ? Je l'ai ! Nino le tire tout doux. Bravo. Tu le mets près de la porte. Le ballon est lisse, un peu poussiéreux. Nino pose le ballon rouge près de la porte. Le parquet craque tout petit. Nino souffle sur le ballon. Un peu de poussière part. Tu as repris le ballon, avant de partir. Il vient au parc. On reprend ses affaires, avant de partir.</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -12092,7 +12626,21 @@
       <c r="AV64" s="2" t="inlineStr"/>
       <c r="AW64" t="inlineStr">
         <is>
-          <t>narrateur|Maya range le ballon, puis cherche encore. Elle reprend ses affaires avant de partir. Un gant manque. Elle le trouve. Maman reste tout près. On va reprendre ses affaires avant de partir.</t>
+          <t>narrateur|Nino est encore dans la chambre.
+narrateur|La chambre sent le savon doux.
+narrateur|Le ballon rouge est sous le lit.
+narrateur|Il touche le deuxième chausson.
+maman|Le ballon, Nino. Tu le reprends ?
+enfant-m|Je l'ai !
+narrateur|Nino le tire tout doux.
+papa|Bravo. Tu le mets près de la porte.
+narrateur|Le ballon est lisse, un peu poussiéreux.
+narrateur|Nino pose le ballon rouge près de la porte.
+narrateur|Le parquet craque tout petit.
+narrateur|Nino souffle sur le ballon. Un peu de poussière part.
+papa|Tu as repris le ballon, avant de partir.
+enfant-m|Il vient au parc.
+maman|On reprend ses affaires, avant de partir.</t>
         </is>
       </c>
       <c r="AX64" t="inlineStr"/>
@@ -12120,7 +12668,7 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre Tom, Léa, ou Sami.</t>
+          <t>Il reste une chose, pour sortir. Le sac, le manteau, ou les chaussures ? Tu choisis, Nino.</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -12288,7 +12836,9 @@
       </c>
       <c r="AW65" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre Tom, Léa, ou Sami.</t>
+          <t>narrateur|Il reste une chose, pour sortir.
+papa|Le sac, le manteau, ou les chaussures ?
+maman|Tu choisis, Nino.</t>
         </is>
       </c>
       <c r="AX65" t="inlineStr"/>
@@ -12316,7 +12866,7 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Maya a choisi la chambre. Puis le ballon rouge. Puis Tom. Le sol est un peu froid. Maya s'assoit près de maman. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>Nino a cherché la chambre. Il a repris le ballon rouge. Maintenant, le sac. Le paillasson est rêche, sous les pieds. Nino ouvre le sac. Il y glisse ce qu'il a repris. Tout est près de la porte. La porte peut s'ouvrir. Bravo. La porte, papa ? Nino reprend ses affaires, avant de partir. On a le seau. On a le manteau. On les prend. On peut sortir. Nino serre ce qu'il tient. Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -12456,10 +13006,26 @@
       <c r="AV66" s="2" t="inlineStr"/>
       <c r="AW66" t="inlineStr">
         <is>
-          <t>narrateur|Maya a choisi la chambre. Puis le ballon rouge. Puis Tom. Le sol est un peu froid. Maya s'assoit près de maman. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
-        </is>
-      </c>
-      <c r="AX66" t="inlineStr"/>
+          <t>narrateur|Nino a cherché la chambre.
+narrateur|Il a repris le ballon rouge.
+narrateur|Maintenant, le sac.
+narrateur|Le paillasson est rêche, sous les pieds.
+narrateur|Nino ouvre le sac. Il y glisse ce qu'il a repris.
+narrateur|Tout est près de la porte.
+papa|La porte peut s'ouvrir. Bravo.
+enfant-m|La porte, papa ?
+narrateur|Nino reprend ses affaires, avant de partir.
+maman|On a le seau. On a le manteau.
+papa|On les prend. On peut sortir.
+narrateur|Nino serre ce qu'il tient.
+enfant-m|Merci, maman. Merci, papa.</t>
+        </is>
+      </c>
+      <c r="AX66" t="inlineStr">
+        <is>
+          <t>porte</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -12484,7 +13050,7 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Papa porte le seau un moment. Nino a repris ses affaires. C'était avant de partir. Bravo, Nino. Tu as fait du bon travail. On va au parc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
@@ -12624,7 +13190,13 @@
       <c r="AV67" s="2" t="inlineStr"/>
       <c r="AW67" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Papa porte le seau un moment.
+narrateur|Nino a repris ses affaires.
+narrateur|C'était avant de partir.
+papa|Bravo, Nino.
+maman|Tu as fait du bon travail.
+enfant-m|On va au parc.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX67" t="inlineStr"/>
@@ -12652,7 +13224,7 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Maya s'arrête près de Léa. le ballon rouge est rangé. Une tasse cliquette. Maya boit une gorgée d'eau. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>Nino a cherché la chambre. Il a repris le ballon rouge. Maintenant, le manteau. La clé de papa tinte dans sa poche. Nino prend le manteau. Il passe un bras, puis l'autre. Tout est près de la porte. Tu as cherché. Tu as pris. Bravo. On y va. Nino reprend ses affaires, avant de partir. On a le seau. On a le manteau. On les prend. On peut sortir. Nino serre ce qu'il tient. Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
@@ -12792,7 +13364,19 @@
       <c r="AV68" s="2" t="inlineStr"/>
       <c r="AW68" t="inlineStr">
         <is>
-          <t>narrateur|Maya s'arrête près de Léa. le ballon rouge est rangé. Une tasse cliquette. Maya boit une gorgée d'eau. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>narrateur|Nino a cherché la chambre.
+narrateur|Il a repris le ballon rouge.
+narrateur|Maintenant, le manteau.
+narrateur|La clé de papa tinte dans sa poche.
+narrateur|Nino prend le manteau. Il passe un bras, puis l'autre.
+narrateur|Tout est près de la porte.
+maman|Tu as cherché. Tu as pris. Bravo.
+enfant-m|On y va.
+narrateur|Nino reprend ses affaires, avant de partir.
+maman|On a le seau. On a le manteau.
+papa|On les prend. On peut sortir.
+narrateur|Nino serre ce qu'il tient.
+enfant-m|Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="AX68" t="inlineStr"/>
@@ -12820,7 +13404,7 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Le doudou est au chaud, sous le manteau. Nino a repris ses affaires. C'était avant de partir. Bravo, Nino. Tu as fait du bon travail. On va au parc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
@@ -12960,7 +13544,13 @@
       <c r="AV69" s="2" t="inlineStr"/>
       <c r="AW69" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Le doudou est au chaud, sous le manteau.
+narrateur|Nino a repris ses affaires.
+narrateur|C'était avant de partir.
+papa|Bravo, Nino.
+maman|Tu as fait du bon travail.
+enfant-m|On va au parc.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX69" t="inlineStr"/>
@@ -12988,7 +13578,7 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Maya se souvient de la chambre. Et de le ballon rouge. Et de Sami. Une chaussette est encore sablée. Maya pose sa tête un moment. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>Nino a cherché la chambre. Il a repris le ballon rouge. Maintenant, les chaussures. Maman plie l'écharpe une dernière fois. Nino enfile les chaussures. Elles font toc toc. Tout est près de la porte. On va au parc. Tes affaires viennent. Le gant est avec moi. Nino reprend ses affaires, avant de partir. On a le seau. On a le manteau. On les prend. On peut sortir. Nino serre ce qu'il tient. Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -13128,7 +13718,19 @@
       <c r="AV70" s="2" t="inlineStr"/>
       <c r="AW70" t="inlineStr">
         <is>
-          <t>narrateur|Maya se souvient de la chambre. Et de le ballon rouge. Et de Sami. Une chaussette est encore sablée. Maya pose sa tête un moment. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>narrateur|Nino a cherché la chambre.
+narrateur|Il a repris le ballon rouge.
+narrateur|Maintenant, les chaussures.
+narrateur|Maman plie l'écharpe une dernière fois.
+narrateur|Nino enfile les chaussures. Elles font toc toc.
+narrateur|Tout est près de la porte.
+papa|On va au parc. Tes affaires viennent.
+enfant-m|Le gant est avec moi.
+narrateur|Nino reprend ses affaires, avant de partir.
+maman|On a le seau. On a le manteau.
+papa|On les prend. On peut sortir.
+narrateur|Nino serre ce qu'il tient.
+enfant-m|Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="AX70" t="inlineStr"/>
@@ -13156,7 +13758,7 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Les affaires de Nino sont avec lui. Nino a repris ses affaires. C'était avant de partir. Bravo, Nino. Tu as fait du bon travail. On va au parc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
@@ -13296,7 +13898,13 @@
       <c r="AV71" s="2" t="inlineStr"/>
       <c r="AW71" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Les affaires de Nino sont avec lui.
+narrateur|Nino a repris ses affaires.
+narrateur|C'était avant de partir.
+papa|Bravo, Nino.
+maman|Tu as fait du bon travail.
+enfant-m|On va au parc.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX71" t="inlineStr"/>
@@ -13324,7 +13932,7 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Maya range le seau, puis cherche encore. Elle reprend ses affaires avant de partir. Un chapeau manque. Elle le trouve. Maman montre le geste, lentement. On va reprendre ses affaires avant de partir.</t>
+          <t>Nino est encore dans la chambre. La chambre sent le savon doux. Le seau bleu sert de coffre, près de l'armoire. Un cube est encore dedans. Le seau, Nino. Tu le reprends avant de partir ? Oui. Et le cube aussi. Nino pose le cube sur l'étagère. Bravo. Tu mets le seau près de la porte. Le seau est sablé, léger. Nino pose le seau bleu près de la porte. Le parquet craque tout petit. Nino tapote le bord du seau. Ça fait toc. Tu as repris le seau, avant de partir. Il vient au parc. On reprend ses affaires, avant de partir.</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -13464,7 +14072,21 @@
       <c r="AV72" s="2" t="inlineStr"/>
       <c r="AW72" t="inlineStr">
         <is>
-          <t>narrateur|Maya range le seau, puis cherche encore. Elle reprend ses affaires avant de partir. Un chapeau manque. Elle le trouve. Maman montre le geste, lentement. On va reprendre ses affaires avant de partir.</t>
+          <t>narrateur|Nino est encore dans la chambre.
+narrateur|La chambre sent le savon doux.
+narrateur|Le seau bleu sert de coffre, près de l'armoire.
+narrateur|Un cube est encore dedans.
+papa|Le seau, Nino. Tu le reprends avant de partir ?
+enfant-m|Oui. Et le cube aussi.
+narrateur|Nino pose le cube sur l'étagère.
+maman|Bravo. Tu mets le seau près de la porte.
+narrateur|Le seau est sablé, léger.
+narrateur|Nino pose le seau bleu près de la porte.
+narrateur|Le parquet craque tout petit.
+narrateur|Nino tapote le bord du seau. Ça fait toc.
+maman|Tu as repris le seau, avant de partir.
+enfant-m|Il vient au parc.
+maman|On reprend ses affaires, avant de partir.</t>
         </is>
       </c>
       <c r="AX72" t="inlineStr"/>
@@ -13492,7 +14114,7 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre Tom, Léa, ou Sami.</t>
+          <t>Il reste une chose, pour sortir. Le sac, le manteau, ou les chaussures ? Tu choisis, Nino.</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
@@ -13660,7 +14282,9 @@
       </c>
       <c r="AW73" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre Tom, Léa, ou Sami.</t>
+          <t>narrateur|Il reste une chose, pour sortir.
+papa|Le sac, le manteau, ou les chaussures ?
+maman|Tu choisis, Nino.</t>
         </is>
       </c>
       <c r="AX73" t="inlineStr"/>
@@ -13688,7 +14312,7 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Avec Tom. Après le seau bleu. Près de la chambre. Maya s'arrête. Un vélo passe au loin. Maya pose le seau bleu à sa place. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>Nino a cherché la chambre. Il a repris le seau bleu. Maintenant, le sac. Le carré de soleil a bougé un peu. Nino ouvre le sac. Il y glisse ce qu'il a repris. Tout est près de la porte. Tu as repris tes affaires, avant de partir. J'ai cherché. Nino reprend ses affaires, avant de partir. On a le seau. On a le manteau. On les prend. On peut sortir. Nino serre ce qu'il tient. Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -13828,10 +14452,26 @@
       <c r="AV74" s="2" t="inlineStr"/>
       <c r="AW74" t="inlineStr">
         <is>
-          <t>narrateur|Avec Tom. Après le seau bleu. Près de la chambre. Maya s'arrête. Un vélo passe au loin. Maya pose le seau bleu à sa place. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
-        </is>
-      </c>
-      <c r="AX74" t="inlineStr"/>
+          <t>narrateur|Nino a cherché la chambre.
+narrateur|Il a repris le seau bleu.
+narrateur|Maintenant, le sac.
+narrateur|Le carré de soleil a bougé un peu.
+narrateur|Nino ouvre le sac. Il y glisse ce qu'il a repris.
+narrateur|Tout est près de la porte.
+maman|Tu as repris tes affaires, avant de partir.
+enfant-m|J'ai cherché.
+narrateur|Nino reprend ses affaires, avant de partir.
+maman|On a le seau. On a le manteau.
+papa|On les prend. On peut sortir.
+narrateur|Nino serre ce qu'il tient.
+enfant-m|Merci, maman. Merci, papa.</t>
+        </is>
+      </c>
+      <c r="AX74" t="inlineStr">
+        <is>
+          <t>porte</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -13856,7 +14496,7 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>La rue est calme, un peu mouillée. Nino a repris ses affaires. C'était avant de partir. Bravo, Nino. Tu as fait du bon travail. On va au parc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -13996,7 +14636,13 @@
       <c r="AV75" s="2" t="inlineStr"/>
       <c r="AW75" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|La rue est calme, un peu mouillée.
+narrateur|Nino a repris ses affaires.
+narrateur|C'était avant de partir.
+papa|Bravo, Nino.
+maman|Tu as fait du bon travail.
+enfant-m|On va au parc.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX75" t="inlineStr"/>
@@ -14024,7 +14670,7 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Maya range le seau bleu. Léa reste près de la chambre. Le savon sent bon. Maya sourit. Maman sourit aussi. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>Nino a cherché la chambre. Il a repris le seau bleu. Maintenant, le manteau. Une miette reste sur la table, loin. Nino prend le manteau. Il passe un bras, puis l'autre. Tout est près de la porte. C'est du bon travail, Nino. C'est bon. Nino reprend ses affaires, avant de partir. On a le seau. On a le manteau. On les prend. On peut sortir. Nino serre ce qu'il tient. Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -14164,7 +14810,19 @@
       <c r="AV76" s="2" t="inlineStr"/>
       <c r="AW76" t="inlineStr">
         <is>
-          <t>narrateur|Maya range le seau bleu. Léa reste près de la chambre. Le savon sent bon. Maya sourit. Maman sourit aussi. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>narrateur|Nino a cherché la chambre.
+narrateur|Il a repris le seau bleu.
+narrateur|Maintenant, le manteau.
+narrateur|Une miette reste sur la table, loin.
+narrateur|Nino prend le manteau. Il passe un bras, puis l'autre.
+narrateur|Tout est près de la porte.
+papa|C'est du bon travail, Nino.
+enfant-m|C'est bon.
+narrateur|Nino reprend ses affaires, avant de partir.
+maman|On a le seau. On a le manteau.
+papa|On les prend. On peut sortir.
+narrateur|Nino serre ce qu'il tient.
+enfant-m|Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="AX76" t="inlineStr"/>
@@ -14192,7 +14850,7 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Nino pose le sac contre sa hanche. Nino a repris ses affaires. C'était avant de partir. Bravo, Nino. Tu as fait du bon travail. On va au parc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
@@ -14332,7 +14990,13 @@
       <c r="AV77" s="2" t="inlineStr"/>
       <c r="AW77" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Nino pose le sac contre sa hanche.
+narrateur|Nino a repris ses affaires.
+narrateur|C'était avant de partir.
+papa|Bravo, Nino.
+maman|Tu as fait du bon travail.
+enfant-m|On va au parc.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX77" t="inlineStr"/>
@@ -14360,7 +15024,7 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Sami est là. le seau bleu aussi. la chambre reste dans le souvenir. Un ballon s'immobilise. Maya ferme la porte, tout doux. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>Nino a cherché la chambre. Il a repris le seau bleu. Maintenant, les chaussures. Le romarin sent fort, par la porte. Nino enfile les chaussures. Elles font toc toc. Tout est près de la porte. Le salon est calme. On peut sortir. Mes affaires, voilà. Nino reprend ses affaires, avant de partir. On a le seau. On a le manteau. On les prend. On peut sortir. Nino serre ce qu'il tient. Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -14500,7 +15164,19 @@
       <c r="AV78" s="2" t="inlineStr"/>
       <c r="AW78" t="inlineStr">
         <is>
-          <t>narrateur|Sami est là. le seau bleu aussi. la chambre reste dans le souvenir. Un ballon s'immobilise. Maya ferme la porte, tout doux. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>narrateur|Nino a cherché la chambre.
+narrateur|Il a repris le seau bleu.
+narrateur|Maintenant, les chaussures.
+narrateur|Le romarin sent fort, par la porte.
+narrateur|Nino enfile les chaussures. Elles font toc toc.
+narrateur|Tout est près de la porte.
+maman|Le salon est calme. On peut sortir.
+enfant-m|Mes affaires, voilà.
+narrateur|Nino reprend ses affaires, avant de partir.
+maman|On a le seau. On a le manteau.
+papa|On les prend. On peut sortir.
+narrateur|Nino serre ce qu'il tient.
+enfant-m|Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="AX78" t="inlineStr"/>
@@ -14528,7 +15204,7 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Le vent est doux, sur les joues. Nino a repris ses affaires. C'était avant de partir. Bravo, Nino. Tu as fait du bon travail. On va au parc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
@@ -14668,7 +15344,13 @@
       <c r="AV79" s="2" t="inlineStr"/>
       <c r="AW79" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Le vent est doux, sur les joues.
+narrateur|Nino a repris ses affaires.
+narrateur|C'était avant de partir.
+papa|Bravo, Nino.
+maman|Tu as fait du bon travail.
+enfant-m|On va au parc.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX79" t="inlineStr"/>
@@ -14696,7 +15378,7 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Maya range le doudou, puis cherche encore. Elle reprend ses affaires avant de partir. Un gant manque. Elle le trouve. Je suis là. On va reprendre ses affaires avant de partir.</t>
+          <t>Nino est encore dans la chambre. La chambre sent le savon doux. Le doudou est dans les draps. Il est encore chaud. Ton doudou, Nino. Tu le reprends ? Oui. Il était au lit. Nino le sort tout doux. Bravo. Tu le mets près de la porte. Le doudou est chaud, un peu froissé. Nino serre le doudou, puis le pose près de la porte. Le parquet craque tout petit. Nino remet l'oreille du doudou à sa place. Tu as repris le doudou, avant de partir. Il vient avec moi. On reprend ses affaires, avant de partir.</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
@@ -14836,8 +15518,21 @@
       <c r="AV80" s="2" t="inlineStr"/>
       <c r="AW80" t="inlineStr">
         <is>
-          <t>narrateur|Maya range le doudou, puis cherche encore. Elle reprend ses affaires avant de partir. Un gant manque. Elle le trouve.
-maman|Je suis là. On va reprendre ses affaires avant de partir.</t>
+          <t>narrateur|Nino est encore dans la chambre.
+narrateur|La chambre sent le savon doux.
+narrateur|Le doudou est dans les draps.
+narrateur|Il est encore chaud.
+maman|Ton doudou, Nino. Tu le reprends ?
+enfant-m|Oui. Il était au lit.
+narrateur|Nino le sort tout doux.
+papa|Bravo. Tu le mets près de la porte.
+narrateur|Le doudou est chaud, un peu froissé.
+narrateur|Nino serre le doudou, puis le pose près de la porte.
+narrateur|Le parquet craque tout petit.
+narrateur|Nino remet l'oreille du doudou à sa place.
+papa|Tu as repris le doudou, avant de partir.
+enfant-m|Il vient avec moi.
+maman|On reprend ses affaires, avant de partir.</t>
         </is>
       </c>
       <c r="AX80" t="inlineStr"/>
@@ -14865,7 +15560,7 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>On peut prendre Tom, Léa, ou Sami.</t>
+          <t>Il reste une chose, pour sortir. Le sac, le manteau, ou les chaussures ? Tu choisis, Nino.</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
@@ -15033,7 +15728,9 @@
       </c>
       <c r="AW81" t="inlineStr">
         <is>
-          <t>narrateur|On peut prendre Tom, Léa, ou Sami.</t>
+          <t>narrateur|Il reste une chose, pour sortir.
+papa|Le sac, le manteau, ou les chaussures ?
+maman|Tu choisis, Nino.</t>
         </is>
       </c>
       <c r="AX81" t="inlineStr"/>
@@ -15061,7 +15758,7 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Maya rejoint Tom. le doudou est rangé. la chambre est fini. On rit un peu. Maya marche près de maman. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>Nino a cherché la chambre. Il a repris le doudou. Maintenant, le sac. Le couloir est frais, tout calme. Nino ouvre le sac. Il y glisse ce qu'il a repris. Tout est près de la porte. Tu tiens bien tes affaires. Bravo. On sort ? Nino reprend ses affaires, avant de partir. On a le seau. On a le manteau. On les prend. On peut sortir. Nino serre ce qu'il tient. Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -15201,10 +15898,26 @@
       <c r="AV82" s="2" t="inlineStr"/>
       <c r="AW82" t="inlineStr">
         <is>
-          <t>narrateur|Maya rejoint Tom. le doudou est rangé. la chambre est fini. On rit un peu. Maya marche près de maman. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
-        </is>
-      </c>
-      <c r="AX82" t="inlineStr"/>
+          <t>narrateur|Nino a cherché la chambre.
+narrateur|Il a repris le doudou.
+narrateur|Maintenant, le sac.
+narrateur|Le couloir est frais, tout calme.
+narrateur|Nino ouvre le sac. Il y glisse ce qu'il a repris.
+narrateur|Tout est près de la porte.
+papa|Tu tiens bien tes affaires. Bravo.
+enfant-m|On sort ?
+narrateur|Nino reprend ses affaires, avant de partir.
+maman|On a le seau. On a le manteau.
+papa|On les prend. On peut sortir.
+narrateur|Nino serre ce qu'il tient.
+enfant-m|Merci, maman. Merci, papa.</t>
+        </is>
+      </c>
+      <c r="AX82" t="inlineStr">
+        <is>
+          <t>porte</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -15229,7 +15942,7 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Le parc attend, tout vert. Nino a repris ses affaires. C'était avant de partir. Bravo, Nino. Tu as fait du bon travail. On va au parc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
@@ -15369,7 +16082,13 @@
       <c r="AV83" s="2" t="inlineStr"/>
       <c r="AW83" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Le parc attend, tout vert.
+narrateur|Nino a repris ses affaires.
+narrateur|C'était avant de partir.
+papa|Bravo, Nino.
+maman|Tu as fait du bon travail.
+enfant-m|On va au parc.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX83" t="inlineStr"/>
@@ -15397,7 +16116,7 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Près de Léa. Maya pose le doudou. la chambre est derrière. L'eau coule, tout petit bruit. Maya range la chambre dans sa tête, comme un souvenir. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>Nino a cherché la chambre. Il a repris le doudou. Maintenant, le manteau. Le coussin du canapé a un creux. Nino prend le manteau. Il passe un bras, puis l'autre. Tout est près de la porte. On est prêts. Merci, Nino. Je tiens bien. Nino reprend ses affaires, avant de partir. On a le seau. On a le manteau. On les prend. On peut sortir. Nino serre ce qu'il tient. Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
@@ -15537,7 +16256,19 @@
       <c r="AV84" s="2" t="inlineStr"/>
       <c r="AW84" t="inlineStr">
         <is>
-          <t>narrateur|Près de Léa. Maya pose le doudou. la chambre est derrière. L'eau coule, tout petit bruit. Maya range la chambre dans sa tête, comme un souvenir. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>narrateur|Nino a cherché la chambre.
+narrateur|Il a repris le doudou.
+narrateur|Maintenant, le manteau.
+narrateur|Le coussin du canapé a un creux.
+narrateur|Nino prend le manteau. Il passe un bras, puis l'autre.
+narrateur|Tout est près de la porte.
+maman|On est prêts. Merci, Nino.
+enfant-m|Je tiens bien.
+narrateur|Nino reprend ses affaires, avant de partir.
+maman|On a le seau. On a le manteau.
+papa|On les prend. On peut sortir.
+narrateur|Nino serre ce qu'il tient.
+enfant-m|Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="AX84" t="inlineStr"/>
@@ -15565,7 +16296,7 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Nino marche près de papa et maman. Nino a repris ses affaires. C'était avant de partir. Bravo, Nino. Tu as fait du bon travail. On va au parc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
@@ -15705,7 +16436,13 @@
       <c r="AV85" s="2" t="inlineStr"/>
       <c r="AW85" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Nino marche près de papa et maman.
+narrateur|Nino a repris ses affaires.
+narrateur|C'était avant de partir.
+papa|Bravo, Nino.
+maman|Tu as fait du bon travail.
+enfant-m|On va au parc.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX85" t="inlineStr"/>
@@ -15733,7 +16470,7 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Maya montre Sami. Maman a vu la chambre. Et le doudou. Un linge sèche à l'air. Maya range encore un peu, près de maman. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>Nino a cherché la chambre. Il a repris le doudou. Maintenant, les chaussures. La vitre a encore une trace brillante. Nino enfile les chaussures. Elles font toc toc. Tout est près de la porte. Avant de partir, tout est repris. Avant de partir, c'est prêt. Nino reprend ses affaires, avant de partir. On a le seau. On a le manteau. On les prend. On peut sortir. Nino serre ce qu'il tient. Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
@@ -15873,7 +16610,19 @@
       <c r="AV86" s="2" t="inlineStr"/>
       <c r="AW86" t="inlineStr">
         <is>
-          <t>narrateur|Maya montre Sami. Maman a vu la chambre. Et le doudou. Un linge sèche à l'air. Maya range encore un peu, près de maman. On va reprendre ses affaires avant de partir. On cherche seau et manteau. On les prend. On va reprendre ses affaires. Maya dit merci à maman.</t>
+          <t>narrateur|Nino a cherché la chambre.
+narrateur|Il a repris le doudou.
+narrateur|Maintenant, les chaussures.
+narrateur|La vitre a encore une trace brillante.
+narrateur|Nino enfile les chaussures. Elles font toc toc.
+narrateur|Tout est près de la porte.
+papa|Avant de partir, tout est repris.
+enfant-m|Avant de partir, c'est prêt.
+narrateur|Nino reprend ses affaires, avant de partir.
+maman|On a le seau. On a le manteau.
+papa|On les prend. On peut sortir.
+narrateur|Nino serre ce qu'il tient.
+enfant-m|Merci, maman. Merci, papa.</t>
         </is>
       </c>
       <c r="AX86" t="inlineStr"/>
@@ -15901,7 +16650,7 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>La maison reste derrière, la porte fermée. Nino a repris ses affaires. C'était avant de partir. Bravo, Nino. Tu as fait du bon travail. On va au parc. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
@@ -16041,7 +16790,13 @@
       <c r="AV87" s="2" t="inlineStr"/>
       <c r="AW87" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|La maison reste derrière, la porte fermée.
+narrateur|Nino a repris ses affaires.
+narrateur|C'était avant de partir.
+papa|Bravo, Nino.
+maman|Tu as fait du bon travail.
+enfant-m|On va au parc.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX87" t="inlineStr"/>
@@ -16063,7 +16818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16157,6 +16912,13 @@
       <c r="A13" t="inlineStr">
         <is>
           <t>F-AUD-007 colonne sons ; vide = silence ; jamais parler dans le bruit</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>F-NAR-009 ouverture du monde, fusion agents</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(F-NAR-019): TREE-AUT-003 polish La tasse de cacao et la vitre
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-AUT-003.xlsx
+++ b/stories/arbres/TREE-AUT-003.xlsx
@@ -2945,17 +2945,17 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Au campement, le soleil de buée tient, rond. Le ballon s'endort contre le mur, miette au chaud. Le crayon rejoint le pot, une pointe un peu humide. Quel moment tu gardes, Mila ? Celui où la goutte est devenue un rayon. La cuillère-étoile a séché, à côté. L'anse bleue fait un dernier toc, tout petit. Dehors, le toit ne goutte plus. J'ai fait le soleil toute seule. Sur le verre, le trait brillant ne glisse plus.</t>
+          <t>Au campement, le soleil de buée tient, rond. Le ballon s'endort contre le mur, miette au chaud. Le crayon rejoint le pot, une pointe un peu humide. Tu as vu le rayon, en bas ? La goutte s'est arrêtée en rayon. La cuillère-étoile a séché, à côté. L'anse bleue fait un dernier toc, tout petit. Dehors, le toit ne goutte plus. J'ai fait le soleil toute seule. Sur le verre, le trait brillant ne glisse plus.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, le soleil de buée tient, rond. Le ballon s'endort contre le mur, miette au chaud. Le crayon rejoint le pot, une pointe un peu humide. Quel moment tu gardes, Mila ? Celui où la &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; est devenue un rayon. La cuillère-étoile a séché, à côté. L'anse bleue fait un dernier toc, tout petit. Dehors, le toit ne goutte plus. J'ai fait le soleil toute seule. Sur le verre, le trait brillant ne glisse plus.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, le soleil de buée tient, rond. Le ballon s'endort contre le mur, miette au chaud. Le crayon rejoint le pot, une pointe un peu humide. Tu as vu le rayon, en bas ? La &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; s'est arrêtée en rayon. La cuillère-étoile a séché, à côté. L'anse bleue fait un dernier toc, tout petit. Dehors, le toit ne goutte plus. J'ai fait le soleil toute seule. Sur le verre, le trait brillant ne glisse plus.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, le soleil de buée tient, rond. Le ballon s'endort contre le mur, miette au chaud. Le crayon rejoint le pot, une pointe un peu humide. Quel moment tu gardes, Mila ? Celui où la &lt;emphasis&gt;goutte&lt;/emphasis&gt; est devenue un rayon. La cuillère-étoile a séché, à côté. L'anse bleue fait un dernier toc, tout petit. Dehors, le toit ne goutte plus. J'ai fait le soleil toute seule. Sur le verre, le trait brillant ne glisse plus.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, le soleil de buée tient, rond. Le ballon s'endort contre le mur, miette au chaud. Le crayon rejoint le pot, une pointe un peu humide. Tu as vu le rayon, en bas ? La &lt;emphasis&gt;goutte&lt;/emphasis&gt; s'est arrêtée en rayon. La cuillère-étoile a séché, à côté. L'anse bleue fait un dernier toc, tout petit. Dehors, le toit ne goutte plus. J'ai fait le soleil toute seule. Sur le verre, le trait brillant ne glisse plus.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -3096,8 +3096,8 @@
           <t>narrateur|Au campement, le soleil de buée tient, rond.
 narrateur|Le ballon s'endort contre le mur, miette au chaud.
 narrateur|Le crayon rejoint le pot, une pointe un peu humide.
-maman|Quel moment tu gardes, Mila ?
-enfant-f|Celui où la goutte est devenue un rayon.
+maman|Tu as vu le rayon, en bas ?
+enfant-f|La goutte s'est arrêtée en rayon.
 papa|La cuillère-étoile a séché, à côté.
 narrateur|L'anse bleue fait un dernier toc, tout petit.
 narrateur|Dehors, le toit ne goutte plus.
@@ -3134,17 +3134,17 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>La tasse n'est plus trop chaude, juste tiède. Je bois un peu. Mon doigt aura chaud. Mila avale. Ça sent le chocolat, tout près. Son doigt, tiède, reprend le rond pâle. Tu traces avec la chaleur, là ? Oui. Le ballon a volé le bruit. Pas le soleil. Le trou se ferme sous la pulpe, sans crayon. L'étoile bleue tape l'anse, tic, contre sa joue. Elle te dit merci, l'étoile ? Elle me dit toc. Le ballon reste loin, sage, la miette au centre. La goutte arrive en bas, et devient un sourire. Nina va goûter, tu crois ? Un tout petit fond. Le reste est pour elle.</t>
+          <t>La tasse n'est plus trop chaude, juste tiède. Je bois un peu. Mon doigt aura chaud. Mila avale. Ça sent le chocolat, tout près. Son doigt, tiède, reprend le rond pâle. Tu traces avec la chaleur, là ? Oui. Le ballon a volé le bruit. Pas le soleil. Le trou se ferme sous la pulpe, sans crayon. L'étoile bleue tape l'anse, tic, contre sa joue. Elle te parle, l'étoile ? Elle me dit toc. Le ballon reste loin, sage, la miette au centre. La goutte arrive en bas, et devient un sourire. Nina va goûter, tu crois ? Un tout petit fond. Le reste est pour elle.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;tasse&lt;/emphasis&gt; n'est plus trop chaude, juste tiède. Je bois un peu. Mon doigt aura chaud. Mila avale. Ça sent le chocolat, tout près. Son doigt, tiède, reprend le rond pâle. Tu traces avec la chaleur, là ? Oui. Le ballon a volé le bruit. Pas le soleil. Le trou se ferme sous la pulpe, sans crayon. L'étoile bleue tape l'anse, tic, contre sa joue. Elle te dit merci, l'étoile ? Elle me dit toc. Le ballon reste loin, sage, la miette au centre. La goutte arrive en bas, et devient un sourire. Nina va goûter, tu crois ? Un tout petit fond. Le reste est pour elle.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;tasse&lt;/emphasis&gt; n'est plus trop chaude, juste tiède. Je bois un peu. Mon doigt aura chaud. Mila avale. Ça sent le chocolat, tout près. Son doigt, tiède, reprend le rond pâle. Tu traces avec la chaleur, là ? Oui. Le ballon a volé le bruit. Pas le soleil. Le trou se ferme sous la pulpe, sans crayon. L'étoile bleue tape l'anse, tic, contre sa joue. Elle te parle, l'étoile ? Elle me dit toc. Le ballon reste loin, sage, la miette au centre. La goutte arrive en bas, et devient un sourire. Nina va goûter, tu crois ? Un tout petit fond. Le reste est pour elle.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>La &lt;emphasis&gt;tasse&lt;/emphasis&gt; n'est plus trop chaude, juste tiède. Je bois un peu. Mon doigt aura chaud. Mila avale. Ça sent le chocolat, tout près. Son doigt, tiède, reprend le rond pâle. Tu traces avec la chaleur, là ? Oui. Le ballon a volé le bruit. Pas le soleil. Le trou se ferme sous la pulpe, sans crayon. L'étoile bleue tape l'anse, tic, contre sa joue. Elle te dit merci, l'étoile ? Elle me dit toc. Le ballon reste loin, sage, la miette au centre. La goutte arrive en bas, et devient un sourire. Nina va goûter, tu crois ? Un tout petit fond. Le reste est pour elle. [pause]</t>
+          <t>La &lt;emphasis&gt;tasse&lt;/emphasis&gt; n'est plus trop chaude, juste tiède. Je bois un peu. Mon doigt aura chaud. Mila avale. Ça sent le chocolat, tout près. Son doigt, tiède, reprend le rond pâle. Tu traces avec la chaleur, là ? Oui. Le ballon a volé le bruit. Pas le soleil. Le trou se ferme sous la pulpe, sans crayon. L'étoile bleue tape l'anse, tic, contre sa joue. Elle te parle, l'étoile ? Elle me dit toc. Le ballon reste loin, sage, la miette au centre. La goutte arrive en bas, et devient un sourire. Nina va goûter, tu crois ? Un tout petit fond. Le reste est pour elle. [pause]</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -3290,7 +3290,7 @@
 enfant-f|Pas le soleil.
 narrateur|Le trou se ferme sous la pulpe, sans crayon.
 narrateur|L'étoile bleue tape l'anse, tic, contre sa joue.
-maman|Elle te dit merci, l'étoile ?
+maman|Elle te parle, l'étoile ?
 enfant-f|Elle me dit toc.
 narrateur|Le ballon reste loin, sage, la miette au centre.
 narrateur|La goutte arrive en bas, et devient un sourire.
@@ -3328,17 +3328,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Au campement, la tasse étoilée a un fond brun. Le ballon s'endort, miette tournée vers la vitre. Le soleil de doigt tient, un peu flou, heureux. Quel moment tu gardes, Mila ? Celui où mon doigt a eu chaud, enfin. La perle jaune de la cuillère brille au sec. Un dernier toc, plus grave, sur la soucoupe. Le tapis tiède garde la forme de ses genoux. J'ai bu, et le soleil est resté. Sur le verre, le sourire de goutte ne bouge plus.</t>
+          <t>Au campement, la tasse étoilée a un fond brun. Le ballon s'endort, miette tournée vers la vitre. Le soleil de doigt tient, un peu flou, heureux. Ton doigt est tiède, maintenant ? Il a tenu le rond, tout seul. La perle jaune de la cuillère brille au sec. Un dernier toc, plus grave, sur la soucoupe. Le tapis tiède garde la forme de ses genoux. J'ai bu, et le soleil est resté. Sur le verre, le sourire de goutte ne bouge plus.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, la tasse étoilée a un fond brun. Le ballon s'endort, miette tournée vers la vitre. Le soleil de doigt tient, un peu flou, heureux. Quel moment tu gardes, Mila ? Celui où mon doigt a eu chaud, enfin. La perle jaune de la cuillère brille au sec. Un dernier toc, plus grave, sur la soucoupe. Le tapis tiède garde la forme de ses genoux. J'ai bu, et le soleil est resté. Sur le verre, le sourire de &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; ne bouge plus.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, la tasse étoilée a un fond brun. Le ballon s'endort, miette tournée vers la vitre. Le soleil de doigt tient, un peu flou, heureux. Ton doigt est tiède, maintenant ? Il a tenu le rond, tout seul. La perle jaune de la cuillère brille au sec. Un dernier toc, plus grave, sur la soucoupe. Le tapis tiède garde la forme de ses genoux. J'ai bu, et le soleil est resté. Sur le verre, le sourire de &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; ne bouge plus.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, la tasse étoilée a un fond brun. Le ballon s'endort, miette tournée vers la vitre. Le soleil de doigt tient, un peu flou, heureux. Quel moment tu gardes, Mila ? Celui où mon doigt a eu chaud, enfin. La perle jaune de la cuillère brille au sec. Un dernier toc, plus grave, sur la soucoupe. Le tapis tiède garde la forme de ses genoux. J'ai bu, et le soleil est resté. Sur le verre, le sourire de &lt;emphasis&gt;goutte&lt;/emphasis&gt; ne bouge plus.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, la tasse étoilée a un fond brun. Le ballon s'endort, miette tournée vers la vitre. Le soleil de doigt tient, un peu flou, heureux. Ton doigt est tiède, maintenant ? Il a tenu le rond, tout seul. La perle jaune de la cuillère brille au sec. Un dernier toc, plus grave, sur la soucoupe. Le tapis tiède garde la forme de ses genoux. J'ai bu, et le soleil est resté. Sur le verre, le sourire de &lt;emphasis&gt;goutte&lt;/emphasis&gt; ne bouge plus.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
@@ -3479,8 +3479,8 @@
           <t>narrateur|Au campement, la tasse étoilée a un fond brun.
 narrateur|Le ballon s'endort, miette tournée vers la vitre.
 narrateur|Le soleil de doigt tient, un peu flou, heureux.
-maman|Quel moment tu gardes, Mila ?
-enfant-f|Celui où mon doigt a eu chaud, enfin.
+maman|Ton doigt est tiède, maintenant ?
+enfant-f|Il a tenu le rond, tout seul.
 papa|La perle jaune de la cuillère brille au sec.
 narrateur|Un dernier toc, plus grave, sur la soucoupe.
 narrateur|Le tapis tiède garde la forme de ses genoux.
@@ -3710,17 +3710,17 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Au campement, l'écharpe sent le cacao, un peu. Le ballon veille au pied, rouge sur le tapis tiède. Le soleil de souffle touche presque le cadre. Quel moment tu gardes, Mila ? Celui où le nuage est revenu, juste pour moi. La cuillère-étoile brille au bord. Un toc étouffé sous la laine, puis le silence. J'ai réchauffé la vitre, toute seule. Sur le verre, le rayon-goutte reste, mince et clair.</t>
+          <t>Au campement, l'écharpe sent le cacao, un peu. Le ballon veille au pied, rouge sur le tapis tiède. Le soleil de souffle touche presque le cadre. Le nuage est revenu, c'est ça ? Il est revenu, juste pour moi. La cuillère-étoile brille au bord. Un toc étouffé sous la laine, puis le silence. J'ai réchauffé la vitre, toute seule. Sur le verre, le rayon-goutte reste, mince et clair.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, l'écharpe sent le cacao, un peu. Le ballon veille au pied, rouge sur le tapis tiède. Le soleil de souffle touche presque le cadre. Quel moment tu gardes, Mila ? Celui où le nuage est revenu, juste pour moi. La cuillère-étoile brille au bord. Un toc étouffé sous la laine, puis le silence. J'ai réchauffé la vitre, toute seule. Sur le verre, le rayon-&lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; reste, mince et clair.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, l'écharpe sent le cacao, un peu. Le ballon veille au pied, rouge sur le tapis tiède. Le soleil de souffle touche presque le cadre. Le nuage est revenu, c'est ça ? Il est revenu, juste pour moi. La cuillère-étoile brille au bord. Un toc étouffé sous la laine, puis le silence. J'ai réchauffé la vitre, toute seule. Sur le verre, le rayon-&lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; reste, mince et clair.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, l'écharpe sent le cacao, un peu. Le ballon veille au pied, rouge sur le tapis tiède. Le soleil de souffle touche presque le cadre. Quel moment tu gardes, Mila ? Celui où le nuage est revenu, juste pour moi. La cuillère-étoile brille au bord. Un toc étouffé sous la laine, puis le silence. J'ai réchauffé la vitre, toute seule. Sur le verre, le rayon-&lt;emphasis&gt;goutte&lt;/emphasis&gt; reste, mince et clair.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, l'écharpe sent le cacao, un peu. Le ballon veille au pied, rouge sur le tapis tiède. Le soleil de souffle touche presque le cadre. Le nuage est revenu, c'est ça ? Il est revenu, juste pour moi. La cuillère-étoile brille au bord. Un toc étouffé sous la laine, puis le silence. J'ai réchauffé la vitre, toute seule. Sur le verre, le rayon-&lt;emphasis&gt;goutte&lt;/emphasis&gt; reste, mince et clair.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr"/>
@@ -3861,8 +3861,8 @@
           <t>narrateur|Au campement, l'écharpe sent le cacao, un peu.
 narrateur|Le ballon veille au pied, rouge sur le tapis tiède.
 narrateur|Le soleil de souffle touche presque le cadre.
-maman|Quel moment tu gardes, Mila ?
-enfant-f|Celui où le nuage est revenu, juste pour moi.
+maman|Le nuage est revenu, c'est ça ?
+enfant-f|Il est revenu, juste pour moi.
 papa|La cuillère-étoile brille au bord.
 narrateur|Un toc étouffé sous la laine, puis le silence.
 enfant-f|J'ai réchauffé la vitre, toute seule.
@@ -4489,17 +4489,17 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Au campement, le soleil habite le haut de la vitre. Le seau bleu, vide, garde une perle d'eau oubliée. Le crayon repose en travers, comme un pont. Quel moment tu gardes, Mila ? Celui où j'ai dessiné au-dessus du flou. La cuillère-étoile a retrouvé son tic. Un toc clair, puis le seau qui ne cloche plus. J'ai sauvé le haut du soleil. Sur le verre, le rayon du haut tient la goutte. Le carrelage a une petite flaque, ronde, sage.</t>
+          <t>Au campement, le soleil habite le haut de la vitre. Le seau bleu, vide, garde une perle d'eau oubliée. Le crayon repose en travers, comme un pont. Tu as dessiné au-dessus du flou ? Le haut du soleil m'a suffi. La cuillère-étoile a retrouvé son tic. Un toc clair, puis le seau qui ne cloche plus. J'ai sauvé le haut du soleil. Sur le verre, le rayon du haut tient la goutte. Le carrelage a une petite flaque, ronde, sage.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, le soleil habite le haut de la vitre. Le seau bleu, vide, garde une perle d'eau oubliée. Le crayon repose en travers, comme un pont. Quel moment tu gardes, Mila ? Celui où j'ai dessiné au-dessus du flou. La cuillère-étoile a retrouvé son tic. Un toc clair, puis le seau qui ne cloche plus. J'ai sauvé le haut du soleil. Sur le verre, le rayon du haut tient la &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt;. Le carrelage a une petite flaque, ronde, sage.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, le soleil habite le haut de la vitre. Le seau bleu, vide, garde une perle d'eau oubliée. Le crayon repose en travers, comme un pont. Tu as dessiné au-dessus du flou ? Le haut du soleil m'a suffi. La cuillère-étoile a retrouvé son tic. Un toc clair, puis le seau qui ne cloche plus. J'ai sauvé le haut du soleil. Sur le verre, le rayon du haut tient la &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt;. Le carrelage a une petite flaque, ronde, sage.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, le soleil habite le haut de la vitre. Le seau bleu, vide, garde une perle d'eau oubliée. Le crayon repose en travers, comme un pont. Quel moment tu gardes, Mila ? Celui où j'ai dessiné au-dessus du flou. La cuillère-étoile a retrouvé son tic. Un toc clair, puis le seau qui ne cloche plus. J'ai sauvé le haut du soleil. Sur le verre, le rayon du haut tient la &lt;emphasis&gt;goutte&lt;/emphasis&gt;. Le carrelage a une petite flaque, ronde, sage.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, le soleil habite le haut de la vitre. Le seau bleu, vide, garde une perle d'eau oubliée. Le crayon repose en travers, comme un pont. Tu as dessiné au-dessus du flou ? Le haut du soleil m'a suffi. La cuillère-étoile a retrouvé son tic. Un toc clair, puis le seau qui ne cloche plus. J'ai sauvé le haut du soleil. Sur le verre, le rayon du haut tient la &lt;emphasis&gt;goutte&lt;/emphasis&gt;. Le carrelage a une petite flaque, ronde, sage.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
@@ -4640,8 +4640,8 @@
           <t>narrateur|Au campement, le soleil habite le haut de la vitre.
 narrateur|Le seau bleu, vide, garde une perle d'eau oubliée.
 narrateur|Le crayon repose en travers, comme un pont.
-maman|Quel moment tu gardes, Mila ?
-enfant-f|Celui où j'ai dessiné au-dessus du flou.
+maman|Tu as dessiné au-dessus du flou ?
+enfant-f|Le haut du soleil m'a suffi.
 papa|La cuillère-étoile a retrouvé son tic.
 narrateur|Un toc clair, puis le seau qui ne cloche plus.
 enfant-f|J'ai sauvé le haut du soleil.
@@ -4872,17 +4872,17 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Au campement, le seau bleu est un plateau d'étoile. La tasse y fait toc, plus grave qu'au début. Le soleil de doigt a un point, en bas, comme un pied. Quel moment tu gardes, Mila ? Celui où le seau a porté à ma place. La perle jaune est sèche, collée au bord. Un toc creux, puis plus rien que le cacao. J'ai bougé la tasse sans la lâcher. Sur le verre, le point-goutte sert de pied au soleil. Le plateau bleu reste, rond, sous l'anse.</t>
+          <t>Au campement, le seau bleu est un plateau d'étoile. La tasse y fait toc, plus grave qu'au début. Le soleil de doigt a un point, en bas, comme un pied. Le seau a porté, vraiment ? Il a porté à ma place. La perle jaune est sèche, collée au bord. Un toc creux, puis plus rien que le cacao. J'ai bougé la tasse sans la lâcher. Sur le verre, le point-goutte sert de pied au soleil. Le plateau bleu reste, rond, sous l'anse.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, le seau bleu est un plateau d'étoile. La tasse y fait toc, plus grave qu'au début. Le soleil de doigt a un point, en bas, comme un pied. Quel moment tu gardes, Mila ? Celui où le seau a porté à ma place. La perle jaune est sèche, collée au bord. Un toc creux, puis plus rien que le cacao. J'ai bougé la tasse sans la lâcher. Sur le verre, le point-&lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; sert de pied au soleil. Le plateau bleu reste, rond, sous l'anse.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, le seau bleu est un plateau d'étoile. La tasse y fait toc, plus grave qu'au début. Le soleil de doigt a un point, en bas, comme un pied. Le seau a porté, vraiment ? Il a porté à ma place. La perle jaune est sèche, collée au bord. Un toc creux, puis plus rien que le cacao. J'ai bougé la tasse sans la lâcher. Sur le verre, le point-&lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; sert de pied au soleil. Le plateau bleu reste, rond, sous l'anse.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, le seau bleu est un plateau d'étoile. La tasse y fait toc, plus grave qu'au début. Le soleil de doigt a un point, en bas, comme un pied. Quel moment tu gardes, Mila ? Celui où le seau a porté à ma place. La perle jaune est sèche, collée au bord. Un toc creux, puis plus rien que le cacao. J'ai bougé la tasse sans la lâcher. Sur le verre, le point-&lt;emphasis&gt;goutte&lt;/emphasis&gt; sert de pied au soleil. Le plateau bleu reste, rond, sous l'anse.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, le seau bleu est un plateau d'étoile. La tasse y fait toc, plus grave qu'au début. Le soleil de doigt a un point, en bas, comme un pied. Le seau a porté, vraiment ? Il a porté à ma place. La perle jaune est sèche, collée au bord. Un toc creux, puis plus rien que le cacao. J'ai bougé la tasse sans la lâcher. Sur le verre, le point-&lt;emphasis&gt;goutte&lt;/emphasis&gt; sert de pied au soleil. Le plateau bleu reste, rond, sous l'anse.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
@@ -5023,8 +5023,8 @@
           <t>narrateur|Au campement, le seau bleu est un plateau d'étoile.
 narrateur|La tasse y fait toc, plus grave qu'au début.
 narrateur|Le soleil de doigt a un point, en bas, comme un pied.
-maman|Quel moment tu gardes, Mila ?
-enfant-f|Celui où le seau a porté à ma place.
+maman|Le seau a porté, vraiment ?
+enfant-f|Il a porté à ma place.
 papa|La perle jaune est sèche, collée au bord.
 narrateur|Un toc creux, puis plus rien que le cacao.
 enfant-f|J'ai bougé la tasse sans la lâcher.
@@ -5252,17 +5252,17 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Au campement, l'écharpe a un coin un peu humide. Le seau bleu, vide, garde l'odeur du bois mouillé. Le soleil de souffle est bas, large, posé. Quel moment tu gardes, Mila ? Celui où la perle a repris son jaune. La cuillère-étoile fait tic, toute sèche. Un toc, puis le froissement de la laine. J'ai séché, puis j'ai dessiné. Sur le verre, le rayon-goutte est large, presque chaud. Le coin d'écharpe sèche près de l'étoile bleue.</t>
+          <t>Au campement, l'écharpe a un coin un peu humide. Le seau bleu, vide, garde l'odeur du bois mouillé. Le soleil de souffle est bas, large, posé. La perle a repris son jaune ? Elle brille, toute sèche. La cuillère-étoile fait tic, toute sèche. Un toc, puis le froissement de la laine. J'ai séché, puis j'ai dessiné. Sur le verre, le rayon-goutte est large, presque chaud. Le coin d'écharpe sèche près de l'étoile bleue.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, l'écharpe a un coin un peu humide. Le seau bleu, vide, garde l'odeur du bois mouillé. Le soleil de souffle est bas, large, posé. Quel moment tu gardes, Mila ? Celui où la perle a repris son jaune. La cuillère-étoile fait tic, toute sèche. Un toc, puis le froissement de la laine. J'ai séché, puis j'ai dessiné. Sur le verre, le rayon-&lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; est large, presque chaud. Le coin d'écharpe sèche près de l'étoile bleue.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, l'écharpe a un coin un peu humide. Le seau bleu, vide, garde l'odeur du bois mouillé. Le soleil de souffle est bas, large, posé. La perle a repris son jaune ? Elle brille, toute sèche. La cuillère-étoile fait tic, toute sèche. Un toc, puis le froissement de la laine. J'ai séché, puis j'ai dessiné. Sur le verre, le rayon-&lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; est large, presque chaud. Le coin d'écharpe sèche près de l'étoile bleue.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, l'écharpe a un coin un peu humide. Le seau bleu, vide, garde l'odeur du bois mouillé. Le soleil de souffle est bas, large, posé. Quel moment tu gardes, Mila ? Celui où la perle a repris son jaune. La cuillère-étoile fait tic, toute sèche. Un toc, puis le froissement de la laine. J'ai séché, puis j'ai dessiné. Sur le verre, le rayon-&lt;emphasis&gt;goutte&lt;/emphasis&gt; est large, presque chaud. Le coin d'écharpe sèche près de l'étoile bleue.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, l'écharpe a un coin un peu humide. Le seau bleu, vide, garde l'odeur du bois mouillé. Le soleil de souffle est bas, large, posé. La perle a repris son jaune ? Elle brille, toute sèche. La cuillère-étoile fait tic, toute sèche. Un toc, puis le froissement de la laine. J'ai séché, puis j'ai dessiné. Sur le verre, le rayon-&lt;emphasis&gt;goutte&lt;/emphasis&gt; est large, presque chaud. Le coin d'écharpe sèche près de l'étoile bleue.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
@@ -5403,8 +5403,8 @@
           <t>narrateur|Au campement, l'écharpe a un coin un peu humide.
 narrateur|Le seau bleu, vide, garde l'odeur du bois mouillé.
 narrateur|Le soleil de souffle est bas, large, posé.
-maman|Quel moment tu gardes, Mila ?
-enfant-f|Celui où la perle a repris son jaune.
+maman|La perle a repris son jaune ?
+enfant-f|Elle brille, toute sèche.
 papa|La cuillère-étoile fait tic, toute sèche.
 narrateur|Un toc, puis le froissement de la laine.
 enfant-f|J'ai séché, puis j'ai dessiné.
@@ -6028,17 +6028,17 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Au campement, le soleil a une étoile au ventre. Le doudou garde son pli en triangle, sage. Le crayon a une pointe un peu de buée. Quel moment tu gardes, Mila ? Celui où l'étoile est allée sur le verre. La cuillère-étoile veille, perle vers le dessin. Un toc, puis plus rien que le tapis tiède. J'ai montré l'anse, sans la cacher. Sur le verre, cinq branches tiennent la goutte. Le triangle de tissu regarde l'étoile vraie.</t>
+          <t>Au campement, le soleil a une étoile au ventre. Le doudou garde son pli en triangle, sage. Le crayon a une pointe un peu de buée. L'étoile est allée sur le verre ? Elle est au centre, pour qu'on la trouve. La cuillère-étoile veille, perle vers le dessin. Un toc, puis plus rien que le tapis tiède. J'ai montré l'anse, sans la cacher. Sur le verre, cinq branches tiennent la goutte. Le triangle de tissu regarde l'étoile vraie.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, le soleil a une étoile au ventre. Le doudou garde son pli en triangle, sage. Le crayon a une pointe un peu de buée. Quel moment tu gardes, Mila ? Celui où l'étoile est allée sur le verre. La cuillère-étoile veille, perle vers le dessin. Un toc, puis plus rien que le tapis tiède. J'ai montré l'anse, sans la cacher. Sur le verre, cinq branches tiennent la &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt;. Le triangle de tissu regarde l'étoile vraie.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, le soleil a une étoile au ventre. Le doudou garde son pli en triangle, sage. Le crayon a une pointe un peu de buée. L'étoile est allée sur le verre ? Elle est au centre, pour qu'on la trouve. La cuillère-étoile veille, perle vers le dessin. Un toc, puis plus rien que le tapis tiède. J'ai montré l'anse, sans la cacher. Sur le verre, cinq branches tiennent la &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt;. Le triangle de tissu regarde l'étoile vraie.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, le soleil a une étoile au ventre. Le doudou garde son pli en triangle, sage. Le crayon a une pointe un peu de buée. Quel moment tu gardes, Mila ? Celui où l'étoile est allée sur le verre. La cuillère-étoile veille, perle vers le dessin. Un toc, puis plus rien que le tapis tiède. J'ai montré l'anse, sans la cacher. Sur le verre, cinq branches tiennent la &lt;emphasis&gt;goutte&lt;/emphasis&gt;. Le triangle de tissu regarde l'étoile vraie.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, le soleil a une étoile au ventre. Le doudou garde son pli en triangle, sage. Le crayon a une pointe un peu de buée. L'étoile est allée sur le verre ? Elle est au centre, pour qu'on la trouve. La cuillère-étoile veille, perle vers le dessin. Un toc, puis plus rien que le tapis tiède. J'ai montré l'anse, sans la cacher. Sur le verre, cinq branches tiennent la &lt;emphasis&gt;goutte&lt;/emphasis&gt;. Le triangle de tissu regarde l'étoile vraie.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -6179,8 +6179,8 @@
           <t>narrateur|Au campement, le soleil a une étoile au ventre.
 narrateur|Le doudou garde son pli en triangle, sage.
 narrateur|Le crayon a une pointe un peu de buée.
-maman|Quel moment tu gardes, Mila ?
-enfant-f|Celui où l'étoile est allée sur le verre.
+maman|L'étoile est allée sur le verre ?
+enfant-f|Elle est au centre, pour qu'on la trouve.
 papa|La cuillère-étoile veille, perle vers le dessin.
 narrateur|Un toc, puis plus rien que le tapis tiède.
 enfant-f|J'ai montré l'anse, sans la cacher.
@@ -6412,17 +6412,17 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Au campement, le doudou est une soucoupe molle. La tasse étoilée y fait un toc mou, content. Le soleil de doigt a un point, sous une étoile. Quel moment tu gardes, Mila ? Celui où le toc est devenu un rire. La cuillère-étoile dort sur le tissu, en travers. Un toc mou, puis l'odeur du savon et du cacao. J'ai bu sans cacher l'anse. Sur le verre, le point-goutte salue l'étoile du milieu. Le nid beige garde un rond un peu plus foncé.</t>
+          <t>Au campement, le doudou est une soucoupe molle. La tasse étoilée y fait un toc mou, content. Le soleil de doigt a un point, sous une étoile. Le toc est devenu un rire ? Un toc mou, comme un rire. La cuillère-étoile dort sur le tissu, en travers. Un toc mou, puis l'odeur du savon et du cacao. J'ai bu sans cacher l'anse. Sur le verre, le point-goutte salue l'étoile du milieu. Le nid beige garde un rond un peu plus foncé.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, le doudou est une soucoupe molle. La tasse étoilée y fait un toc mou, content. Le soleil de doigt a un point, sous une étoile. Quel moment tu gardes, Mila ? Celui où le toc est devenu un rire. La cuillère-étoile dort sur le tissu, en travers. Un toc mou, puis l'odeur du savon et du cacao. J'ai bu sans cacher l'anse. Sur le verre, le point-&lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; salue l'étoile du milieu. Le nid beige garde un rond un peu plus foncé.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, le doudou est une soucoupe molle. La tasse étoilée y fait un toc mou, content. Le soleil de doigt a un point, sous une étoile. Le toc est devenu un rire ? Un toc mou, comme un rire. La cuillère-étoile dort sur le tissu, en travers. Un toc mou, puis l'odeur du savon et du cacao. J'ai bu sans cacher l'anse. Sur le verre, le point-&lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; salue l'étoile du milieu. Le nid beige garde un rond un peu plus foncé.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, le doudou est une soucoupe molle. La tasse étoilée y fait un toc mou, content. Le soleil de doigt a un point, sous une étoile. Quel moment tu gardes, Mila ? Celui où le toc est devenu un rire. La cuillère-étoile dort sur le tissu, en travers. Un toc mou, puis l'odeur du savon et du cacao. J'ai bu sans cacher l'anse. Sur le verre, le point-&lt;emphasis&gt;goutte&lt;/emphasis&gt; salue l'étoile du milieu. Le nid beige garde un rond un peu plus foncé.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, le doudou est une soucoupe molle. La tasse étoilée y fait un toc mou, content. Le soleil de doigt a un point, sous une étoile. Le toc est devenu un rire ? Un toc mou, comme un rire. La cuillère-étoile dort sur le tissu, en travers. Un toc mou, puis l'odeur du savon et du cacao. J'ai bu sans cacher l'anse. Sur le verre, le point-&lt;emphasis&gt;goutte&lt;/emphasis&gt; salue l'étoile du milieu. Le nid beige garde un rond un peu plus foncé.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
@@ -6563,8 +6563,8 @@
           <t>narrateur|Au campement, le doudou est une soucoupe molle.
 narrateur|La tasse étoilée y fait un toc mou, content.
 narrateur|Le soleil de doigt a un point, sous une étoile.
-maman|Quel moment tu gardes, Mila ?
-enfant-f|Celui où le toc est devenu un rire.
+maman|Le toc est devenu un rire ?
+enfant-f|Un toc mou, comme un rire.
 papa|La cuillère-étoile dort sur le tissu, en travers.
 narrateur|Un toc mou, puis l'odeur du savon et du cacao.
 enfant-f|J'ai bu sans cacher l'anse.
@@ -6796,17 +6796,17 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Au campement, deux tissus gardent la tasse étoilée. L'étoile bleue reste dehors, ronde, visible. Le soleil de souffle est large, presque un manteau. Quel moment tu gardes, Mila ? Celui où l'anse a eu le droit d'être vue. La cuillère-étoile dépasse, perle vers la vitre. Un toc net, puis le silence des deux laines. J'ai soufflé, sans cacher l'étoile. Sur le verre, le rayon-goutte touche un pli d'écharpe. Le coin de doudou garde la forme de l'anse.</t>
+          <t>Au campement, deux tissus gardent la tasse étoilée. L'étoile bleue reste dehors, ronde, visible. Le soleil de souffle est large, presque un manteau. L'anse a eu le droit d'être vue ? Dehors, pour le toc, et pour Nina. La cuillère-étoile dépasse, perle vers la vitre. Un toc net, puis le silence des deux laines. J'ai soufflé, sans cacher l'étoile. Sur le verre, le rayon-goutte touche un pli d'écharpe. Le coin de doudou garde la forme de l'anse.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, deux tissus gardent la tasse étoilée. L'étoile bleue reste dehors, ronde, visible. Le soleil de souffle est large, presque un manteau. Quel moment tu gardes, Mila ? Celui où l'anse a eu le droit d'être vue. La cuillère-étoile dépasse, perle vers la vitre. Un toc net, puis le silence des deux laines. J'ai soufflé, sans cacher l'étoile. Sur le verre, le rayon-&lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; touche un pli d'écharpe. Le coin de doudou garde la forme de l'anse.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, deux tissus gardent la tasse étoilée. L'étoile bleue reste dehors, ronde, visible. Le soleil de souffle est large, presque un manteau. L'anse a eu le droit d'être vue ? Dehors, pour le toc, et pour Nina. La cuillère-étoile dépasse, perle vers la vitre. Un toc net, puis le silence des deux laines. J'ai soufflé, sans cacher l'étoile. Sur le verre, le rayon-&lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; touche un pli d'écharpe. Le coin de doudou garde la forme de l'anse.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, deux tissus gardent la tasse étoilée. L'étoile bleue reste dehors, ronde, visible. Le soleil de souffle est large, presque un manteau. Quel moment tu gardes, Mila ? Celui où l'anse a eu le droit d'être vue. La cuillère-étoile dépasse, perle vers la vitre. Un toc net, puis le silence des deux laines. J'ai soufflé, sans cacher l'étoile. Sur le verre, le rayon-&lt;emphasis&gt;goutte&lt;/emphasis&gt; touche un pli d'écharpe. Le coin de doudou garde la forme de l'anse.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, deux tissus gardent la tasse étoilée. L'étoile bleue reste dehors, ronde, visible. Le soleil de souffle est large, presque un manteau. L'anse a eu le droit d'être vue ? Dehors, pour le toc, et pour Nina. La cuillère-étoile dépasse, perle vers la vitre. Un toc net, puis le silence des deux laines. J'ai soufflé, sans cacher l'étoile. Sur le verre, le rayon-&lt;emphasis&gt;goutte&lt;/emphasis&gt; touche un pli d'écharpe. Le coin de doudou garde la forme de l'anse.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
@@ -6947,8 +6947,8 @@
           <t>narrateur|Au campement, deux tissus gardent la tasse étoilée.
 narrateur|L'étoile bleue reste dehors, ronde, visible.
 narrateur|Le soleil de souffle est large, presque un manteau.
-maman|Quel moment tu gardes, Mila ?
-enfant-f|Celui où l'anse a eu le droit d'être vue.
+maman|L'anse a eu le droit d'être vue ?
+enfant-f|Dehors, pour le toc, et pour Nina.
 papa|La cuillère-étoile dépasse, perle vers la vitre.
 narrateur|Un toc net, puis le silence des deux laines.
 enfant-f|J'ai soufflé, sans cacher l'étoile.
@@ -8337,17 +8337,17 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Au campement, deux gouttes se tiennent par un trait. Le ballon, sec, garde un rond plus pâle au flanc. Le crayon sent la menthe, un peu, à la pointe. Quel moment tu gardes, Mila ? Celui où le dedans a parlé au dehors. La feuille de menthe a séché, en virgule. Un toc, puis une dalle qui ne claque plus. J'ai rendu la goutte au soleil. Sur le verre, le pont mince ne glisse plus. Le passage des gouttes, dehors, s'est tu.</t>
+          <t>Au campement, deux gouttes se tiennent par un trait. Le ballon, sec, garde un rond plus pâle au flanc. Le crayon sent la menthe, un peu, à la pointe. Le dedans a parlé au dehors ? Les deux gouttes se tiennent. La feuille de menthe a séché, en virgule. Un toc, puis une dalle qui ne claque plus. J'ai rendu la goutte au soleil. Sur le verre, le pont mince ne glisse plus. Le passage des gouttes, dehors, s'est tu.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, deux &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt;s se tiennent par un trait. Le ballon, sec, garde un rond plus pâle au flanc. Le crayon sent la menthe, un peu, à la pointe. Quel moment tu gardes, Mila ? Celui où le dedans a parlé au dehors. La feuille de menthe a séché, en virgule. Un toc, puis une dalle qui ne claque plus. J'ai rendu la goutte au soleil. Sur le verre, le pont mince ne glisse plus. Le passage des gouttes, dehors, s'est tu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, deux &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt;s se tiennent par un trait. Le ballon, sec, garde un rond plus pâle au flanc. Le crayon sent la menthe, un peu, à la pointe. Le dedans a parlé au dehors ? Les deux gouttes se tiennent. La feuille de menthe a séché, en virgule. Un toc, puis une dalle qui ne claque plus. J'ai rendu la goutte au soleil. Sur le verre, le pont mince ne glisse plus. Le passage des gouttes, dehors, s'est tu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, deux &lt;emphasis&gt;goutte&lt;/emphasis&gt;s se tiennent par un trait. Le ballon, sec, garde un rond plus pâle au flanc. Le crayon sent la menthe, un peu, à la pointe. Quel moment tu gardes, Mila ? Celui où le dedans a parlé au dehors. La feuille de menthe a séché, en virgule. Un toc, puis une dalle qui ne claque plus. J'ai rendu la goutte au soleil. Sur le verre, le pont mince ne glisse plus. Le passage des gouttes, dehors, s'est tu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, deux &lt;emphasis&gt;goutte&lt;/emphasis&gt;s se tiennent par un trait. Le ballon, sec, garde un rond plus pâle au flanc. Le crayon sent la menthe, un peu, à la pointe. Le dedans a parlé au dehors ? Les deux gouttes se tiennent. La feuille de menthe a séché, en virgule. Un toc, puis une dalle qui ne claque plus. J'ai rendu la goutte au soleil. Sur le verre, le pont mince ne glisse plus. Le passage des gouttes, dehors, s'est tu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr"/>
@@ -8488,8 +8488,8 @@
           <t>narrateur|Au campement, deux gouttes se tiennent par un trait.
 narrateur|Le ballon, sec, garde un rond plus pâle au flanc.
 narrateur|Le crayon sent la menthe, un peu, à la pointe.
-maman|Quel moment tu gardes, Mila ?
-enfant-f|Celui où le dedans a parlé au dehors.
+maman|Le dedans a parlé au dehors ?
+enfant-f|Les deux gouttes se tiennent.
 papa|La feuille de menthe a séché, en virgule.
 narrateur|Un toc, puis une dalle qui ne claque plus.
 enfant-f|J'ai rendu la goutte au soleil.
@@ -8722,17 +8722,17 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Au campement, le cacao sent la menthe, enfin. Le ballon, sec, tourne sa trace vers la porte. Le soleil de doigt a un point frais, comme une dalle. Quel moment tu gardes, Mila ? Celui où le nez a trouvé le jardin. La feuille flotte, petite barque, dans le fond. Un toc, puis l'odeur verte qui ne part plus. J'ai bu le dehors, sans ouvrir. Sur le verre, le point-goutte est plus clair que les autres. Le paillasson garde un rond de ballon, presque sec.</t>
+          <t>Au campement, le cacao sent la menthe, enfin. Le ballon, sec, tourne sa trace vers la porte. Le soleil de doigt a un point frais, comme une dalle. Le nez a trouvé le jardin ? La menthe, avant les yeux. La feuille flotte, petite barque, dans le fond. Un toc, puis l'odeur verte qui ne part plus. J'ai bu le dehors, sans ouvrir. Sur le verre, le point-goutte est plus clair que les autres. Le paillasson garde un rond de ballon, presque sec.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, le cacao sent la menthe, enfin. Le ballon, sec, tourne sa trace vers la porte. Le soleil de doigt a un point frais, comme une dalle. Quel moment tu gardes, Mila ? Celui où le nez a trouvé le jardin. La feuille flotte, petite barque, dans le fond. Un toc, puis l'odeur verte qui ne part plus. J'ai bu le dehors, sans ouvrir. Sur le verre, le point-&lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; est plus clair que les autres. Le paillasson garde un rond de ballon, presque sec.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, le cacao sent la menthe, enfin. Le ballon, sec, tourne sa trace vers la porte. Le soleil de doigt a un point frais, comme une dalle. Le nez a trouvé le jardin ? La menthe, avant les yeux. La feuille flotte, petite barque, dans le fond. Un toc, puis l'odeur verte qui ne part plus. J'ai bu le dehors, sans ouvrir. Sur le verre, le point-&lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; est plus clair que les autres. Le paillasson garde un rond de ballon, presque sec.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, le cacao sent la menthe, enfin. Le ballon, sec, tourne sa trace vers la porte. Le soleil de doigt a un point frais, comme une dalle. Quel moment tu gardes, Mila ? Celui où le nez a trouvé le jardin. La feuille flotte, petite barque, dans le fond. Un toc, puis l'odeur verte qui ne part plus. J'ai bu le dehors, sans ouvrir. Sur le verre, le point-&lt;emphasis&gt;goutte&lt;/emphasis&gt; est plus clair que les autres. Le paillasson garde un rond de ballon, presque sec.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, le cacao sent la menthe, enfin. Le ballon, sec, tourne sa trace vers la porte. Le soleil de doigt a un point frais, comme une dalle. Le nez a trouvé le jardin ? La menthe, avant les yeux. La feuille flotte, petite barque, dans le fond. Un toc, puis l'odeur verte qui ne part plus. J'ai bu le dehors, sans ouvrir. Sur le verre, le point-&lt;emphasis&gt;goutte&lt;/emphasis&gt; est plus clair que les autres. Le paillasson garde un rond de ballon, presque sec.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr"/>
@@ -8873,8 +8873,8 @@
           <t>narrateur|Au campement, le cacao sent la menthe, enfin.
 narrateur|Le ballon, sec, tourne sa trace vers la porte.
 narrateur|Le soleil de doigt a un point frais, comme une dalle.
-maman|Quel moment tu gardes, Mila ?
-enfant-f|Celui où le nez a trouvé le jardin.
+maman|Le nez a trouvé le jardin ?
+enfant-f|La menthe, avant les yeux.
 papa|La feuille flotte, petite barque, dans le fond.
 narrateur|Un toc, puis l'odeur verte qui ne part plus.
 enfant-f|J'ai bu le dehors, sans ouvrir.
@@ -9106,17 +9106,17 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Au campement, le soleil a une menthe au cœur. L'écharpe sent l'air du passage des gouttes. Le ballon, sec, n'a plus de miroir au flanc. Quel moment tu gardes, Mila ? Celui où la feuille a laissé son peigne. La vraie menthe sèche, à côté, un peu froissée. Un toc, puis un froissement d'écharpe. J'ai tamponné le dehors sur le dedans. Sur le verre, une dent de menthe tient la goutte. Le paillasson ne brille plus.</t>
+          <t>Au campement, le soleil a une menthe au cœur. L'écharpe sent l'air du passage des gouttes. Le ballon, sec, n'a plus de miroir au flanc. La feuille a laissé son peigne ? Un tampon de menthe, au milieu. La vraie menthe sèche, à côté, un peu froissée. Un toc, puis un froissement d'écharpe. J'ai tamponné le dehors sur le dedans. Sur le verre, une dent de menthe tient la goutte. Le paillasson ne brille plus.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, le soleil a une menthe au cœur. L'écharpe sent l'air du passage des &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt;s. Le ballon, sec, n'a plus de miroir au flanc. Quel moment tu gardes, Mila ? Celui où la feuille a laissé son peigne. La vraie menthe sèche, à côté, un peu froissée. Un toc, puis un froissement d'écharpe. J'ai tamponné le dehors sur le dedans. Sur le verre, une dent de menthe tient la goutte. Le paillasson ne brille plus.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, le soleil a une menthe au cœur. L'écharpe sent l'air du passage des &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt;s. Le ballon, sec, n'a plus de miroir au flanc. La feuille a laissé son peigne ? Un tampon de menthe, au milieu. La vraie menthe sèche, à côté, un peu froissée. Un toc, puis un froissement d'écharpe. J'ai tamponné le dehors sur le dedans. Sur le verre, une dent de menthe tient la goutte. Le paillasson ne brille plus.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, le soleil a une menthe au cœur. L'écharpe sent l'air du passage des &lt;emphasis&gt;goutte&lt;/emphasis&gt;s. Le ballon, sec, n'a plus de miroir au flanc. Quel moment tu gardes, Mila ? Celui où la feuille a laissé son peigne. La vraie menthe sèche, à côté, un peu froissée. Un toc, puis un froissement d'écharpe. J'ai tamponné le dehors sur le dedans. Sur le verre, une dent de menthe tient la goutte. Le paillasson ne brille plus.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, le soleil a une menthe au cœur. L'écharpe sent l'air du passage des &lt;emphasis&gt;goutte&lt;/emphasis&gt;s. Le ballon, sec, n'a plus de miroir au flanc. La feuille a laissé son peigne ? Un tampon de menthe, au milieu. La vraie menthe sèche, à côté, un peu froissée. Un toc, puis un froissement d'écharpe. J'ai tamponné le dehors sur le dedans. Sur le verre, une dent de menthe tient la goutte. Le paillasson ne brille plus.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
@@ -9257,8 +9257,8 @@
           <t>narrateur|Au campement, le soleil a une menthe au cœur.
 narrateur|L'écharpe sent l'air du passage des gouttes.
 narrateur|Le ballon, sec, n'a plus de miroir au flanc.
-maman|Quel moment tu gardes, Mila ?
-enfant-f|Celui où la feuille a laissé son peigne.
+maman|La feuille a laissé son peigne ?
+enfant-f|Un tampon de menthe, au milieu.
 papa|La vraie menthe sèche, à côté, un peu froissée.
 narrateur|Un toc, puis un froissement d'écharpe.
 enfant-f|J'ai tamponné le dehors sur le dedans.
@@ -9884,17 +9884,17 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Au campement, une rivière de buée monte vers un soleil. Le seau bleu garde une perle, rien qu'une. Le crayon a le bois un peu taché de vert. Quel moment tu gardes, Mila ? Celui où l'eau est devenue un chemin. La menthe, sur le bord, a la forme d'un bateau. Un toc sec, puis plus de cloche dans le seau. J'ai dessiné ce que l'eau avait emporté. Sur le verre, la rivière tient la goutte au milieu. Le passage des gouttes, dehors, est terne, fini.</t>
+          <t>Au campement, une rivière de buée monte vers un soleil. Le seau bleu garde une perle, rien qu'une. Le crayon a le bois un peu taché de vert. L'eau est devenue un chemin ? Une rivière, du seau au soleil. La menthe, sur le bord, a la forme d'un bateau. Un toc sec, puis plus de cloche dans le seau. J'ai dessiné ce que l'eau avait emporté. Sur le verre, la rivière tient la goutte au milieu. Le passage des gouttes, dehors, est terne, fini.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, une rivière de buée monte vers un soleil. Le seau bleu garde une perle, rien qu'une. Le crayon a le bois un peu taché de vert. Quel moment tu gardes, Mila ? Celui où l'eau est devenue un chemin. La menthe, sur le bord, a la forme d'un bateau. Un toc sec, puis plus de cloche dans le seau. J'ai dessiné ce que l'eau avait emporté. Sur le verre, la rivière tient la &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; au milieu. Le passage des gouttes, dehors, est terne, fini.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, une rivière de buée monte vers un soleil. Le seau bleu garde une perle, rien qu'une. Le crayon a le bois un peu taché de vert. L'eau est devenue un chemin ? Une rivière, du seau au soleil. La menthe, sur le bord, a la forme d'un bateau. Un toc sec, puis plus de cloche dans le seau. J'ai dessiné ce que l'eau avait emporté. Sur le verre, la rivière tient la &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; au milieu. Le passage des gouttes, dehors, est terne, fini.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, une rivière de buée monte vers un soleil. Le seau bleu garde une perle, rien qu'une. Le crayon a le bois un peu taché de vert. Quel moment tu gardes, Mila ? Celui où l'eau est devenue un chemin. La menthe, sur le bord, a la forme d'un bateau. Un toc sec, puis plus de cloche dans le seau. J'ai dessiné ce que l'eau avait emporté. Sur le verre, la rivière tient la &lt;emphasis&gt;goutte&lt;/emphasis&gt; au milieu. Le passage des gouttes, dehors, est terne, fini.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, une rivière de buée monte vers un soleil. Le seau bleu garde une perle, rien qu'une. Le crayon a le bois un peu taché de vert. L'eau est devenue un chemin ? Une rivière, du seau au soleil. La menthe, sur le bord, a la forme d'un bateau. Un toc sec, puis plus de cloche dans le seau. J'ai dessiné ce que l'eau avait emporté. Sur le verre, la rivière tient la &lt;emphasis&gt;goutte&lt;/emphasis&gt; au milieu. Le passage des gouttes, dehors, est terne, fini.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr"/>
@@ -10035,8 +10035,8 @@
           <t>narrateur|Au campement, une rivière de buée monte vers un soleil.
 narrateur|Le seau bleu garde une perle, rien qu'une.
 narrateur|Le crayon a le bois un peu taché de vert.
-maman|Quel moment tu gardes, Mila ?
-enfant-f|Celui où l'eau est devenue un chemin.
+maman|L'eau est devenue un chemin ?
+enfant-f|Une rivière, du seau au soleil.
 papa|La menthe, sur le bord, a la forme d'un bateau.
 narrateur|Un toc sec, puis plus de cloche dans le seau.
 enfant-f|J'ai dessiné ce que l'eau avait emporté.
@@ -10268,17 +10268,17 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Au campement, le seau bleu est une table de tasse. Le cacao sent une menthe discrète, revenue. Le soleil de doigt a une perle, jumelle du seau. Quel moment tu gardes, Mila ? Celui où les deux perles se sont vues. La feuille a coulé, puis elle flotte, petite. Un toc grave, creux, comme un puits gentil. J'ai rendu l'odeur, sans l'eau de trop. Sur le verre, la perle-goutte ne glisse plus. Le seau, table, ne cloche plus.</t>
+          <t>Au campement, le seau bleu est une table de tasse. Le cacao sent une menthe discrète, revenue. Le soleil de doigt a une perle, jumelle du seau. Les deux perles se sont vues ? Une dans le seau, une sur le verre. La feuille a coulé, puis elle flotte, petite. Un toc grave, creux, comme un puits gentil. J'ai rendu l'odeur, sans l'eau de trop. Sur le verre, la perle-goutte ne glisse plus. Le seau, table, ne cloche plus.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, le seau bleu est une table de tasse. Le cacao sent une menthe discrète, revenue. Le soleil de doigt a une perle, jumelle du seau. Quel moment tu gardes, Mila ? Celui où les deux perles se sont vues. La feuille a coulé, puis elle flotte, petite. Un toc grave, creux, comme un puits gentil. J'ai rendu l'odeur, sans l'eau de trop. Sur le verre, la perle-&lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; ne glisse plus. Le seau, table, ne cloche plus.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, le seau bleu est une table de tasse. Le cacao sent une menthe discrète, revenue. Le soleil de doigt a une perle, jumelle du seau. Les deux perles se sont vues ? Une dans le seau, une sur le verre. La feuille a coulé, puis elle flotte, petite. Un toc grave, creux, comme un puits gentil. J'ai rendu l'odeur, sans l'eau de trop. Sur le verre, la perle-&lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; ne glisse plus. Le seau, table, ne cloche plus.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, le seau bleu est une table de tasse. Le cacao sent une menthe discrète, revenue. Le soleil de doigt a une perle, jumelle du seau. Quel moment tu gardes, Mila ? Celui où les deux perles se sont vues. La feuille a coulé, puis elle flotte, petite. Un toc grave, creux, comme un puits gentil. J'ai rendu l'odeur, sans l'eau de trop. Sur le verre, la perle-&lt;emphasis&gt;goutte&lt;/emphasis&gt; ne glisse plus. Le seau, table, ne cloche plus.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, le seau bleu est une table de tasse. Le cacao sent une menthe discrète, revenue. Le soleil de doigt a une perle, jumelle du seau. Les deux perles se sont vues ? Une dans le seau, une sur le verre. La feuille a coulé, puis elle flotte, petite. Un toc grave, creux, comme un puits gentil. J'ai rendu l'odeur, sans l'eau de trop. Sur le verre, la perle-&lt;emphasis&gt;goutte&lt;/emphasis&gt; ne glisse plus. Le seau, table, ne cloche plus.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
@@ -10419,8 +10419,8 @@
           <t>narrateur|Au campement, le seau bleu est une table de tasse.
 narrateur|Le cacao sent une menthe discrète, revenue.
 narrateur|Le soleil de doigt a une perle, jumelle du seau.
-maman|Quel moment tu gardes, Mila ?
-enfant-f|Celui où les deux perles se sont vues.
+maman|Les deux perles se sont vues ?
+enfant-f|Une dans le seau, une sur le verre.
 papa|La feuille a coulé, puis elle flotte, petite.
 narrateur|Un toc grave, creux, comme un puits gentil.
 enfant-f|J'ai rendu l'odeur, sans l'eau de trop.
@@ -10651,17 +10651,17 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Au campement, un soleil entoure une ombre de menthe. L'écharpe sent l'air froid, arrêté à la porte. Le seau bleu cale le bois, vide et utile. Quel moment tu gardes, Mila ? Celui où l'ombre de la feuille est devenue un cœur. La vraie menthe sèche, collée au bord, en virgule. Un toc, puis plus d'air froid sur les chevilles. J'ai tenu le jardin à sa place. Sur le verre, l'ombre-goutte est verte pour de faux. La porte ne claque plus.</t>
+          <t>Au campement, un soleil entoure une ombre de menthe. L'écharpe sent l'air froid, arrêté à la porte. Le seau bleu cale le bois, vide et utile. L'ombre est devenue un cœur ? L'ombre de la feuille, au centre. La vraie menthe sèche, collée au bord, en virgule. Un toc, puis plus d'air froid sur les chevilles. J'ai tenu le jardin à sa place. Sur le verre, l'ombre-goutte est verte pour de faux. La porte ne claque plus.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, un soleil entoure une ombre de menthe. L'écharpe sent l'air froid, arrêté à la porte. Le seau bleu cale le bois, vide et utile. Quel moment tu gardes, Mila ? Celui où l'ombre de la feuille est devenue un cœur. La vraie menthe sèche, collée au bord, en virgule. Un toc, puis plus d'air froid sur les chevilles. J'ai tenu le jardin à sa place. Sur le verre, l'ombre-&lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; est verte pour de faux. La porte ne claque plus.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, un soleil entoure une ombre de menthe. L'écharpe sent l'air froid, arrêté à la porte. Le seau bleu cale le bois, vide et utile. L'ombre est devenue un cœur ? L'ombre de la feuille, au centre. La vraie menthe sèche, collée au bord, en virgule. Un toc, puis plus d'air froid sur les chevilles. J'ai tenu le jardin à sa place. Sur le verre, l'ombre-&lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; est verte pour de faux. La porte ne claque plus.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, un soleil entoure une ombre de menthe. L'écharpe sent l'air froid, arrêté à la porte. Le seau bleu cale le bois, vide et utile. Quel moment tu gardes, Mila ? Celui où l'ombre de la feuille est devenue un cœur. La vraie menthe sèche, collée au bord, en virgule. Un toc, puis plus d'air froid sur les chevilles. J'ai tenu le jardin à sa place. Sur le verre, l'ombre-&lt;emphasis&gt;goutte&lt;/emphasis&gt; est verte pour de faux. La porte ne claque plus.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, un soleil entoure une ombre de menthe. L'écharpe sent l'air froid, arrêté à la porte. Le seau bleu cale le bois, vide et utile. L'ombre est devenue un cœur ? L'ombre de la feuille, au centre. La vraie menthe sèche, collée au bord, en virgule. Un toc, puis plus d'air froid sur les chevilles. J'ai tenu le jardin à sa place. Sur le verre, l'ombre-&lt;emphasis&gt;goutte&lt;/emphasis&gt; est verte pour de faux. La porte ne claque plus.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr"/>
@@ -10802,8 +10802,8 @@
           <t>narrateur|Au campement, un soleil entoure une ombre de menthe.
 narrateur|L'écharpe sent l'air froid, arrêté à la porte.
 narrateur|Le seau bleu cale le bois, vide et utile.
-maman|Quel moment tu gardes, Mila ?
-enfant-f|Celui où l'ombre de la feuille est devenue un cœur.
+maman|L'ombre est devenue un cœur ?
+enfant-f|L'ombre de la feuille, au centre.
 papa|La vraie menthe sèche, collée au bord, en virgule.
 narrateur|Un toc, puis plus d'air froid sur les chevilles.
 enfant-f|J'ai tenu le jardin à sa place.
@@ -11429,17 +11429,17 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Au campement, un nuage denté entoure un soleil. Le doudou montre une médaille verte, presque sèche. Le crayon a une pointe un peu jardin. Quel moment tu gardes, Mila ? Celui où la tache est devenue un nuage. La menthe vraie sèche, loin du tissu. Un toc net, puis plus de dalle derrière la porte. J'ai changé la tache en dessin. Sur le verre, l'ovale tient la goutte comme un nid. La médaille du doudou ne s'étend plus.</t>
+          <t>Au campement, un nuage denté entoure un soleil. Le doudou montre une médaille verte, presque sèche. Le crayon a une pointe un peu jardin. La tache est devenue un nuage ? Un ovale denté, plus une saleté. La menthe vraie sèche, loin du tissu. Un toc net, puis plus de dalle derrière la porte. J'ai changé la tache en dessin. Sur le verre, l'ovale tient la goutte comme un nid. La médaille du doudou ne s'étend plus.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, un nuage denté entoure un soleil. Le doudou montre une médaille verte, presque sèche. Le crayon a une pointe un peu jardin. Quel moment tu gardes, Mila ? Celui où la tache est devenue un nuage. La menthe vraie sèche, loin du tissu. Un toc net, puis plus de dalle derrière la porte. J'ai changé la tache en dessin. Sur le verre, l'ovale tient la &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; comme un nid. La médaille du doudou ne s'étend plus.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, un nuage denté entoure un soleil. Le doudou montre une médaille verte, presque sèche. Le crayon a une pointe un peu jardin. La tache est devenue un nuage ? Un ovale denté, plus une saleté. La menthe vraie sèche, loin du tissu. Un toc net, puis plus de dalle derrière la porte. J'ai changé la tache en dessin. Sur le verre, l'ovale tient la &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; comme un nid. La médaille du doudou ne s'étend plus.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, un nuage denté entoure un soleil. Le doudou montre une médaille verte, presque sèche. Le crayon a une pointe un peu jardin. Quel moment tu gardes, Mila ? Celui où la tache est devenue un nuage. La menthe vraie sèche, loin du tissu. Un toc net, puis plus de dalle derrière la porte. J'ai changé la tache en dessin. Sur le verre, l'ovale tient la &lt;emphasis&gt;goutte&lt;/emphasis&gt; comme un nid. La médaille du doudou ne s'étend plus.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, un nuage denté entoure un soleil. Le doudou montre une médaille verte, presque sèche. Le crayon a une pointe un peu jardin. La tache est devenue un nuage ? Un ovale denté, plus une saleté. La menthe vraie sèche, loin du tissu. Un toc net, puis plus de dalle derrière la porte. J'ai changé la tache en dessin. Sur le verre, l'ovale tient la &lt;emphasis&gt;goutte&lt;/emphasis&gt; comme un nid. La médaille du doudou ne s'étend plus.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
@@ -11580,8 +11580,8 @@
           <t>narrateur|Au campement, un nuage denté entoure un soleil.
 narrateur|Le doudou montre une médaille verte, presque sèche.
 narrateur|Le crayon a une pointe un peu jardin.
-maman|Quel moment tu gardes, Mila ?
-enfant-f|Celui où la tache est devenue un nuage.
+maman|La tache est devenue un nuage ?
+enfant-f|Un ovale denté, plus une saleté.
 papa|La menthe vraie sèche, loin du tissu.
 narrateur|Un toc net, puis plus de dalle derrière la porte.
 enfant-f|J'ai changé la tache en dessin.
@@ -11815,17 +11815,17 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Au campement, le cacao sent la menthe et le savon. Le doudou tourne sa médaille vers le mur, discrète. Le soleil de doigt a un point, loin de tout vert. Quel moment tu gardes, Mila ? Celui où l'étoile a regardé toute seule. La feuille de menthe sèche, à l'écart du tissu. Un toc clair, sans laine par-dessus. J'ai bu, et le doudou a eu sa place. Sur le verre, le point-goutte est loin de la tache. Le beige du doudou redevient le plus visible.</t>
+          <t>Au campement, le cacao sent la menthe et le savon. Le doudou tourne sa médaille vers le mur, discrète. Le soleil de doigt a un point, loin de tout vert. L'étoile a regardé toute seule ? Le bleu vers la vitre, le vert caché. La feuille de menthe sèche, à l'écart du tissu. Un toc clair, sans laine par-dessus. J'ai bu, et le doudou a eu sa place. Sur le verre, le point-goutte est loin de la tache. Le beige du doudou redevient le plus visible.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, le cacao sent la menthe et le savon. Le doudou tourne sa médaille vers le mur, discrète. Le soleil de doigt a un point, loin de tout vert. Quel moment tu gardes, Mila ? Celui où l'étoile a regardé toute seule. La feuille de menthe sèche, à l'écart du tissu. Un toc clair, sans laine par-dessus. J'ai bu, et le doudou a eu sa place. Sur le verre, le point-&lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; est loin de la tache. Le beige du doudou redevient le plus visible.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, le cacao sent la menthe et le savon. Le doudou tourne sa médaille vers le mur, discrète. Le soleil de doigt a un point, loin de tout vert. L'étoile a regardé toute seule ? Le bleu vers la vitre, le vert caché. La feuille de menthe sèche, à l'écart du tissu. Un toc clair, sans laine par-dessus. J'ai bu, et le doudou a eu sa place. Sur le verre, le point-&lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; est loin de la tache. Le beige du doudou redevient le plus visible.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, le cacao sent la menthe et le savon. Le doudou tourne sa médaille vers le mur, discrète. Le soleil de doigt a un point, loin de tout vert. Quel moment tu gardes, Mila ? Celui où l'étoile a regardé toute seule. La feuille de menthe sèche, à l'écart du tissu. Un toc clair, sans laine par-dessus. J'ai bu, et le doudou a eu sa place. Sur le verre, le point-&lt;emphasis&gt;goutte&lt;/emphasis&gt; est loin de la tache. Le beige du doudou redevient le plus visible.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, le cacao sent la menthe et le savon. Le doudou tourne sa médaille vers le mur, discrète. Le soleil de doigt a un point, loin de tout vert. L'étoile a regardé toute seule ? Le bleu vers la vitre, le vert caché. La feuille de menthe sèche, à l'écart du tissu. Un toc clair, sans laine par-dessus. J'ai bu, et le doudou a eu sa place. Sur le verre, le point-&lt;emphasis&gt;goutte&lt;/emphasis&gt; est loin de la tache. Le beige du doudou redevient le plus visible.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr"/>
@@ -11966,8 +11966,8 @@
           <t>narrateur|Au campement, le cacao sent la menthe et le savon.
 narrateur|Le doudou tourne sa médaille vers le mur, discrète.
 narrateur|Le soleil de doigt a un point, loin de tout vert.
-maman|Quel moment tu gardes, Mila ?
-enfant-f|Celui où l'étoile a regardé toute seule.
+maman|L'étoile a regardé toute seule ?
+enfant-f|Le bleu vers la vitre, le vert caché.
 papa|La feuille de menthe sèche, à l'écart du tissu.
 narrateur|Un toc clair, sans laine par-dessus.
 enfant-f|J'ai bu, et le doudou a eu sa place.
@@ -12201,17 +12201,17 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Au campement, deux ronds de buée se regardent. L'écharpe sent le passage des gouttes, arrêté. Le doudou s'abrite sous l'ovale, médaille cachée. Quel moment tu gardes, Mila ? Celui où le doudou a eu son propre soleil. La menthe sèche entre les deux dessins, en bas. Un toc net, puis deux silences de laine. J'ai soufflé pour deux. Sur le verre, la goutte habite le plus grand rond. L'ovale du doudou, lui, reste vide et fier.</t>
+          <t>Au campement, deux ronds de buée se regardent. L'écharpe sent le passage des gouttes, arrêté. Le doudou s'abrite sous l'ovale, médaille cachée. Le doudou a eu son soleil ? Un petit rond, rien que pour lui. La menthe sèche entre les deux dessins, en bas. Un toc net, puis deux silences de laine. J'ai soufflé pour deux. Sur le verre, la goutte habite le plus grand rond. L'ovale du doudou, lui, reste vide et fier.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, deux ronds de buée se regardent. L'écharpe sent le passage des &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt;s, arrêté. Le doudou s'abrite sous l'ovale, médaille cachée. Quel moment tu gardes, Mila ? Celui où le doudou a eu son propre soleil. La menthe sèche entre les deux dessins, en bas. Un toc net, puis deux silences de laine. J'ai soufflé pour deux. Sur le verre, la goutte habite le plus grand rond. L'ovale du doudou, lui, reste vide et fier.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, deux ronds de buée se regardent. L'écharpe sent le passage des &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt;s, arrêté. Le doudou s'abrite sous l'ovale, médaille cachée. Le doudou a eu son soleil ? Un petit rond, rien que pour lui. La menthe sèche entre les deux dessins, en bas. Un toc net, puis deux silences de laine. J'ai soufflé pour deux. Sur le verre, la goutte habite le plus grand rond. L'ovale du doudou, lui, reste vide et fier.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, deux ronds de buée se regardent. L'écharpe sent le passage des &lt;emphasis&gt;goutte&lt;/emphasis&gt;s, arrêté. Le doudou s'abrite sous l'ovale, médaille cachée. Quel moment tu gardes, Mila ? Celui où le doudou a eu son propre soleil. La menthe sèche entre les deux dessins, en bas. Un toc net, puis deux silences de laine. J'ai soufflé pour deux. Sur le verre, la goutte habite le plus grand rond. L'ovale du doudou, lui, reste vide et fier.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, deux ronds de buée se regardent. L'écharpe sent le passage des &lt;emphasis&gt;goutte&lt;/emphasis&gt;s, arrêté. Le doudou s'abrite sous l'ovale, médaille cachée. Le doudou a eu son soleil ? Un petit rond, rien que pour lui. La menthe sèche entre les deux dessins, en bas. Un toc net, puis deux silences de laine. J'ai soufflé pour deux. Sur le verre, la goutte habite le plus grand rond. L'ovale du doudou, lui, reste vide et fier.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr"/>
@@ -12352,8 +12352,8 @@
           <t>narrateur|Au campement, deux ronds de buée se regardent.
 narrateur|L'écharpe sent le passage des gouttes, arrêté.
 narrateur|Le doudou s'abrite sous l'ovale, médaille cachée.
-maman|Quel moment tu gardes, Mila ?
-enfant-f|Celui où le doudou a eu son propre soleil.
+maman|Le doudou a eu son soleil ?
+enfant-f|Un petit rond, rien que pour lui.
 papa|La menthe sèche entre les deux dessins, en bas.
 narrateur|Un toc net, puis deux silences de laine.
 enfant-f|J'ai soufflé pour deux.
@@ -12390,17 +12390,17 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Mila entre dans la chambre, trop pressée. Le nid de laine est un tas de couvertures. Le carré beige cache son bord sous l'oreiller. Pour tenir la tasse, sans me brûler. Elle fouille. Un chausson tombe, puis un livre. Pas de carré. Ses mains se ferment, vides. Il a disparu. Sous l'oreiller, peut-être ? Mila soulève l'oreiller. Le carré est là, tiède. Et la tasse étoilée ? Elle est restée au salon. Elle revient, le carré contre la poitrine. Tu la reprends ? Oui. J'ai besoin d'elle.</t>
+          <t>Mila entre dans la chambre, trop pressée. Le nid de laine est un tas de couvertures. Le carré beige cache son bord sous l'oreiller. Pour tenir la tasse, au chaud. Elle fouille. Un chausson tombe, puis un livre. Pas de carré. Ses mains se ferment, vides. Il a disparu. Sous l'oreiller, peut-être ? Mila soulève l'oreiller. Le carré est là, tiède. Et la tasse étoilée ? Elle est restée au salon. Elle revient, le carré contre la poitrine. Tu la reprends ? Oui. J'ai besoin d'elle.</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila entre dans la chambre, trop pressée. Le nid de laine est un tas de couvertures. Le carré beige cache son bord sous l'oreiller. Pour tenir la tasse, sans me brûler. Elle fouille. Un chausson tombe, puis un livre. Pas de carré. Ses mains se ferment, vides. Il a disparu. Sous l'oreiller, peut-être ? Mila soulève l'oreiller. Le carré est là, tiède. Et la tasse étoilée ? Elle est restée au salon. Elle revient, le carré contre la poitrine. Tu la reprends ? Oui. J'ai besoin d'elle.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila entre dans la chambre, trop pressée. Le nid de laine est un tas de couvertures. Le carré beige cache son bord sous l'oreiller. Pour tenir la tasse, au chaud. Elle fouille. Un chausson tombe, puis un livre. Pas de carré. Ses mains se ferment, vides. Il a disparu. Sous l'oreiller, peut-être ? Mila soulève l'oreiller. Le carré est là, tiède. Et la tasse étoilée ? Elle est restée au salon. Elle revient, le carré contre la poitrine. Tu la reprends ? Oui. J'ai besoin d'elle.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Mila entre dans la chambre, trop pressée. Le nid de laine est un tas de couvertures. Le carré beige cache son bord sous l'oreiller. Pour tenir la tasse, sans me brûler. Elle fouille. Un chausson tombe, puis un livre. Pas de carré. Ses mains se ferment, vides. Il a disparu. Sous l'oreiller, peut-être ? Mila soulève l'oreiller. Le carré est là, tiède. Et la tasse étoilée ? Elle est restée au salon. Elle revient, le carré contre la poitrine. Tu la reprends ? Oui. J'ai besoin d'elle. [pause]</t>
+          <t>Mila entre dans la chambre, trop pressée. Le nid de laine est un tas de couvertures. Le carré beige cache son bord sous l'oreiller. Pour tenir la tasse, au chaud. Elle fouille. Un chausson tombe, puis un livre. Pas de carré. Ses mains se ferment, vides. Il a disparu. Sous l'oreiller, peut-être ? Mila soulève l'oreiller. Le carré est là, tiède. Et la tasse étoilée ? Elle est restée au salon. Elle revient, le carré contre la poitrine. Tu la reprends ? Oui. J'ai besoin d'elle. [pause]</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr"/>
@@ -12537,7 +12537,7 @@
           <t>narrateur|Mila entre dans la chambre, trop pressée.
 narrateur|Le nid de laine est un tas de couvertures.
 narrateur|Le carré beige cache son bord sous l'oreiller.
-enfant-f|Pour tenir la tasse, sans me brûler.
+enfant-f|Pour tenir la tasse, au chaud.
 narrateur|Elle fouille.
 narrateur|Un chausson tombe, puis un livre.
 narrateur|Pas de carré.
@@ -13746,17 +13746,17 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Au campement, une spirale de buée noue un soleil. Le ballon, sous la chaise, n'a plus de fil. Le crayon a une pointe un peu laineuse, pour de faux. Quel moment tu gardes, Mila ? Celui où le fil est devenu un nœud sur le verre. Le vrai fil dort dans ta poche, en boucle. Un toc clair, sous le carré de laine. J'ai donné un manteau au soleil. Sur le verre, la goutte habite la boucle, sans glisser. Le nid de la chambre, loin, s'est tu.</t>
+          <t>Au campement, une spirale de buée noue un soleil. Le ballon, sous la chaise, n'a plus de fil. Le crayon a une pointe un peu laineuse, pour de faux. Le fil est devenu un nœud ? Une boucle de buée, en haut. Le vrai fil dort dans ta poche, en boucle. Un toc clair, sous le carré de laine. J'ai donné un manteau au soleil. Sur le verre, la goutte habite la boucle, sans glisser. Le nid de la chambre, loin, s'est tu.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, une spirale de buée noue un soleil. Le ballon, sous la chaise, n'a plus de fil. Le crayon a une pointe un peu laineuse, pour de faux. Quel moment tu gardes, Mila ? Celui où le fil est devenu un nœud sur le verre. Le vrai fil dort dans ta poche, en boucle. Un toc clair, sous le carré de laine. J'ai donné un manteau au soleil. Sur le verre, la &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; habite la boucle, sans glisser. Le nid de la chambre, loin, s'est tu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, une spirale de buée noue un soleil. Le ballon, sous la chaise, n'a plus de fil. Le crayon a une pointe un peu laineuse, pour de faux. Le fil est devenu un nœud ? Une boucle de buée, en haut. Le vrai fil dort dans ta poche, en boucle. Un toc clair, sous le carré de laine. J'ai donné un manteau au soleil. Sur le verre, la &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; habite la boucle, sans glisser. Le nid de la chambre, loin, s'est tu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, une spirale de buée noue un soleil. Le ballon, sous la chaise, n'a plus de fil. Le crayon a une pointe un peu laineuse, pour de faux. Quel moment tu gardes, Mila ? Celui où le fil est devenu un nœud sur le verre. Le vrai fil dort dans ta poche, en boucle. Un toc clair, sous le carré de laine. J'ai donné un manteau au soleil. Sur le verre, la &lt;emphasis&gt;goutte&lt;/emphasis&gt; habite la boucle, sans glisser. Le nid de la chambre, loin, s'est tu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, une spirale de buée noue un soleil. Le ballon, sous la chaise, n'a plus de fil. Le crayon a une pointe un peu laineuse, pour de faux. Le fil est devenu un nœud ? Une boucle de buée, en haut. Le vrai fil dort dans ta poche, en boucle. Un toc clair, sous le carré de laine. J'ai donné un manteau au soleil. Sur le verre, la &lt;emphasis&gt;goutte&lt;/emphasis&gt; habite la boucle, sans glisser. Le nid de la chambre, loin, s'est tu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr"/>
@@ -13897,8 +13897,8 @@
           <t>narrateur|Au campement, une spirale de buée noue un soleil.
 narrateur|Le ballon, sous la chaise, n'a plus de fil.
 narrateur|Le crayon a une pointe un peu laineuse, pour de faux.
-maman|Quel moment tu gardes, Mila ?
-enfant-f|Celui où le fil est devenu un nœud sur le verre.
+maman|Le fil est devenu un nœud ?
+enfant-f|Une boucle de buée, en haut.
 papa|Le vrai fil dort dans ta poche, en boucle.
 narrateur|Un toc clair, sous le carré de laine.
 enfant-f|J'ai donné un manteau au soleil.
@@ -14131,17 +14131,17 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Au campement, le carré de laine est une anse molle. Le ballon dort sous la chaise, sans fil. Le soleil de doigt a un point chaud, beige pour de faux. Quel moment tu gardes, Mila ? Celui où l'anse est restée visible, malgré le chaud. Le fil, dans ta poche, ne s'échappe plus. Un toc doux, juste, sous la laine. J'ai bu sans tout couvrir. Sur le verre, le point-goutte a la couleur du carré. L'oreiller de la chambre a gardé un creux, vide.</t>
+          <t>Au campement, le carré de laine est une anse molle. Le ballon dort sous la chaise, sans fil. Le soleil de doigt a un point chaud, beige pour de faux. L'anse est restée visible ? Un coin, malgré le chaud. Le fil, dans ta poche, ne s'échappe plus. Un toc doux, juste, sous la laine. J'ai bu sans tout couvrir. Sur le verre, le point-goutte a la couleur du carré. L'oreiller de la chambre a gardé un creux, vide.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, le carré de laine est une anse molle. Le ballon dort sous la chaise, sans fil. Le soleil de doigt a un point chaud, beige pour de faux. Quel moment tu gardes, Mila ? Celui où l'anse est restée visible, malgré le chaud. Le fil, dans ta poche, ne s'échappe plus. Un toc doux, juste, sous la laine. J'ai bu sans tout couvrir. Sur le verre, le point-&lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; a la couleur du carré. L'oreiller de la chambre a gardé un creux, vide.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, le carré de laine est une anse molle. Le ballon dort sous la chaise, sans fil. Le soleil de doigt a un point chaud, beige pour de faux. L'anse est restée visible ? Un coin, malgré le chaud. Le fil, dans ta poche, ne s'échappe plus. Un toc doux, juste, sous la laine. J'ai bu sans tout couvrir. Sur le verre, le point-&lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; a la couleur du carré. L'oreiller de la chambre a gardé un creux, vide.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, le carré de laine est une anse molle. Le ballon dort sous la chaise, sans fil. Le soleil de doigt a un point chaud, beige pour de faux. Quel moment tu gardes, Mila ? Celui où l'anse est restée visible, malgré le chaud. Le fil, dans ta poche, ne s'échappe plus. Un toc doux, juste, sous la laine. J'ai bu sans tout couvrir. Sur le verre, le point-&lt;emphasis&gt;goutte&lt;/emphasis&gt; a la couleur du carré. L'oreiller de la chambre a gardé un creux, vide.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, le carré de laine est une anse molle. Le ballon dort sous la chaise, sans fil. Le soleil de doigt a un point chaud, beige pour de faux. L'anse est restée visible ? Un coin, malgré le chaud. Le fil, dans ta poche, ne s'échappe plus. Un toc doux, juste, sous la laine. J'ai bu sans tout couvrir. Sur le verre, le point-&lt;emphasis&gt;goutte&lt;/emphasis&gt; a la couleur du carré. L'oreiller de la chambre a gardé un creux, vide.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr"/>
@@ -14282,8 +14282,8 @@
           <t>narrateur|Au campement, le carré de laine est une anse molle.
 narrateur|Le ballon dort sous la chaise, sans fil.
 narrateur|Le soleil de doigt a un point chaud, beige pour de faux.
-maman|Quel moment tu gardes, Mila ?
-enfant-f|Celui où l'anse est restée visible, malgré le chaud.
+maman|L'anse est restée visible ?
+enfant-f|Un coin, malgré le chaud.
 papa|Le fil, dans ta poche, ne s'échappe plus.
 narrateur|Un toc doux, juste, sous la laine.
 enfant-f|J'ai bu sans tout couvrir.
@@ -14516,17 +14516,17 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Au campement, deux laines gardent un toc étouffé. L'étoile bleue a une fenêtre, ronde, dans le tissu. Le soleil de souffle est large, presque une couverture. Quel moment tu gardes, Mila ? Celui où l'anse a eu une fenêtre, pas un cache. Le ballon, sous la chaise, n'a plus rien à voler. Un toc étouffé, puis le silence des laines. J'ai soufflé avec deux chauds. Sur le verre, le rayon-goutte est le plus large. Le fil, dans la poche, fait une boule sage.</t>
+          <t>Au campement, deux laines gardent un toc étouffé. L'étoile bleue a une fenêtre, ronde, dans le tissu. Le soleil de souffle est large, presque une couverture. L'anse a eu une fenêtre ? Une fenêtre ronde, pas un cache. Le ballon, sous la chaise, n'a plus rien à voler. Un toc étouffé, puis le silence des laines. J'ai soufflé avec deux chauds. Sur le verre, le rayon-goutte est le plus large. Le fil, dans la poche, fait une boule sage.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, deux laines gardent un toc étouffé. L'étoile bleue a une fenêtre, ronde, dans le tissu. Le soleil de souffle est large, presque une couverture. Quel moment tu gardes, Mila ? Celui où l'anse a eu une fenêtre, pas un cache. Le ballon, sous la chaise, n'a plus rien à voler. Un toc étouffé, puis le silence des laines. J'ai soufflé avec deux chauds. Sur le verre, le rayon-&lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; est le plus large. Le fil, dans la poche, fait une boule sage.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, deux laines gardent un toc étouffé. L'étoile bleue a une fenêtre, ronde, dans le tissu. Le soleil de souffle est large, presque une couverture. L'anse a eu une fenêtre ? Une fenêtre ronde, pas un cache. Le ballon, sous la chaise, n'a plus rien à voler. Un toc étouffé, puis le silence des laines. J'ai soufflé avec deux chauds. Sur le verre, le rayon-&lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; est le plus large. Le fil, dans la poche, fait une boule sage.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, deux laines gardent un toc étouffé. L'étoile bleue a une fenêtre, ronde, dans le tissu. Le soleil de souffle est large, presque une couverture. Quel moment tu gardes, Mila ? Celui où l'anse a eu une fenêtre, pas un cache. Le ballon, sous la chaise, n'a plus rien à voler. Un toc étouffé, puis le silence des laines. J'ai soufflé avec deux chauds. Sur le verre, le rayon-&lt;emphasis&gt;goutte&lt;/emphasis&gt; est le plus large. Le fil, dans la poche, fait une boule sage.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, deux laines gardent un toc étouffé. L'étoile bleue a une fenêtre, ronde, dans le tissu. Le soleil de souffle est large, presque une couverture. L'anse a eu une fenêtre ? Une fenêtre ronde, pas un cache. Le ballon, sous la chaise, n'a plus rien à voler. Un toc étouffé, puis le silence des laines. J'ai soufflé avec deux chauds. Sur le verre, le rayon-&lt;emphasis&gt;goutte&lt;/emphasis&gt; est le plus large. Le fil, dans la poche, fait une boule sage.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr"/>
@@ -14667,8 +14667,8 @@
           <t>narrateur|Au campement, deux laines gardent un toc étouffé.
 narrateur|L'étoile bleue a une fenêtre, ronde, dans le tissu.
 narrateur|Le soleil de souffle est large, presque une couverture.
-maman|Quel moment tu gardes, Mila ?
-enfant-f|Celui où l'anse a eu une fenêtre, pas un cache.
+maman|L'anse a eu une fenêtre ?
+enfant-f|Une fenêtre ronde, pas un cache.
 papa|Le ballon, sous la chaise, n'a plus rien à voler.
 narrateur|Un toc étouffé, puis le silence des laines.
 enfant-f|J'ai soufflé avec deux chauds.
@@ -15299,17 +15299,17 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Au campement, deux mains de buée tiennent un soleil. Le seau bleu, vide, a de la place, enfin. Le crayon a tracé des doigts un peu trop grands. Quel moment tu gardes, Mila ? Celui où mes mains n'ont plus été trop pleines. Le chausson dort sous le lit, à sa place. Un toc net, rien qui penche. J'ai dessiné le un par un. Sur le verre, la goutte habite l'espace entre deux doigts. La commode, loin, n'a plus la tasse.</t>
+          <t>Au campement, deux mains de buée tiennent un soleil. Le seau bleu, vide, a de la place, enfin. Le crayon a tracé des doigts un peu trop grands. Tes mains n'étaient plus trop pleines ? Une chose, puis l'autre. Le chausson dort sous le lit, à sa place. Un toc net, rien qui penche. J'ai dessiné le un par un. Sur le verre, la goutte habite l'espace entre deux doigts. La commode, loin, n'a plus la tasse.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, deux mains de buée tiennent un soleil. Le seau bleu, vide, a de la place, enfin. Le crayon a tracé des doigts un peu trop grands. Quel moment tu gardes, Mila ? Celui où mes mains n'ont plus été trop pleines. Le chausson dort sous le lit, à sa place. Un toc net, rien qui penche. J'ai dessiné le un par un. Sur le verre, la &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; habite l'espace entre deux doigts. La commode, loin, n'a plus la tasse.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, deux mains de buée tiennent un soleil. Le seau bleu, vide, a de la place, enfin. Le crayon a tracé des doigts un peu trop grands. Tes mains n'étaient plus trop pleines ? Une chose, puis l'autre. Le chausson dort sous le lit, à sa place. Un toc net, rien qui penche. J'ai dessiné le un par un. Sur le verre, la &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; habite l'espace entre deux doigts. La commode, loin, n'a plus la tasse.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, deux mains de buée tiennent un soleil. Le seau bleu, vide, a de la place, enfin. Le crayon a tracé des doigts un peu trop grands. Quel moment tu gardes, Mila ? Celui où mes mains n'ont plus été trop pleines. Le chausson dort sous le lit, à sa place. Un toc net, rien qui penche. J'ai dessiné le un par un. Sur le verre, la &lt;emphasis&gt;goutte&lt;/emphasis&gt; habite l'espace entre deux doigts. La commode, loin, n'a plus la tasse.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, deux mains de buée tiennent un soleil. Le seau bleu, vide, a de la place, enfin. Le crayon a tracé des doigts un peu trop grands. Tes mains n'étaient plus trop pleines ? Une chose, puis l'autre. Le chausson dort sous le lit, à sa place. Un toc net, rien qui penche. J'ai dessiné le un par un. Sur le verre, la &lt;emphasis&gt;goutte&lt;/emphasis&gt; habite l'espace entre deux doigts. La commode, loin, n'a plus la tasse.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr"/>
@@ -15450,8 +15450,8 @@
           <t>narrateur|Au campement, deux mains de buée tiennent un soleil.
 narrateur|Le seau bleu, vide, a de la place, enfin.
 narrateur|Le crayon a tracé des doigts un peu trop grands.
-maman|Quel moment tu gardes, Mila ?
-enfant-f|Celui où mes mains n'ont plus été trop pleines.
+maman|Tes mains n'étaient plus trop pleines ?
+enfant-f|Une chose, puis l'autre.
 papa|Le chausson dort sous le lit, à sa place.
 narrateur|Un toc net, rien qui penche.
 enfant-f|J'ai dessiné le un par un.
@@ -15689,17 +15689,17 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Au campement, trois étages : seau, laine, étoile. Le soleil de doigt a un point, pile au centre. La tasse étoilée a le toc le plus petit, le juste. Quel moment tu gardes, Mila ? Celui des trois tocs, de plus en plus vrais. Le chausson n'est plus dans le seau. Un dernier petit toc, puis le cacao. J'ai mis l'ordre, pas la chambre. Sur le verre, le point-goutte est au centre du rond. La commode est vide, et ça va.</t>
+          <t>Au campement, trois étages : seau, laine, étoile. Le soleil de doigt a un point, pile au centre. La tasse étoilée a le toc le plus petit, le juste. Les trois tocs étaient justes ? De plus en plus vrais, un par un. Le chausson n'est plus dans le seau. Un dernier petit toc, puis le cacao. J'ai mis l'ordre, pas la chambre. Sur le verre, le point-goutte est au centre du rond. La commode est vide, et ça va.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, trois étages : seau, laine, étoile. Le soleil de doigt a un point, pile au centre. La tasse étoilée a le toc le plus petit, le juste. Quel moment tu gardes, Mila ? Celui des trois tocs, de plus en plus vrais. Le chausson n'est plus dans le seau. Un dernier petit toc, puis le cacao. J'ai mis l'ordre, pas la chambre. Sur le verre, le point-&lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; est au centre du rond. La commode est vide, et ça va.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, trois étages : seau, laine, étoile. Le soleil de doigt a un point, pile au centre. La tasse étoilée a le toc le plus petit, le juste. Les trois tocs étaient justes ? De plus en plus vrais, un par un. Le chausson n'est plus dans le seau. Un dernier petit toc, puis le cacao. J'ai mis l'ordre, pas la chambre. Sur le verre, le point-&lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; est au centre du rond. La commode est vide, et ça va.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, trois étages : seau, laine, étoile. Le soleil de doigt a un point, pile au centre. La tasse étoilée a le toc le plus petit, le juste. Quel moment tu gardes, Mila ? Celui des trois tocs, de plus en plus vrais. Le chausson n'est plus dans le seau. Un dernier petit toc, puis le cacao. J'ai mis l'ordre, pas la chambre. Sur le verre, le point-&lt;emphasis&gt;goutte&lt;/emphasis&gt; est au centre du rond. La commode est vide, et ça va.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, trois étages : seau, laine, étoile. Le soleil de doigt a un point, pile au centre. La tasse étoilée a le toc le plus petit, le juste. Les trois tocs étaient justes ? De plus en plus vrais, un par un. Le chausson n'est plus dans le seau. Un dernier petit toc, puis le cacao. J'ai mis l'ordre, pas la chambre. Sur le verre, le point-&lt;emphasis&gt;goutte&lt;/emphasis&gt; est au centre du rond. La commode est vide, et ça va.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr"/>
@@ -15840,8 +15840,8 @@
           <t>narrateur|Au campement, trois étages : seau, laine, étoile.
 narrateur|Le soleil de doigt a un point, pile au centre.
 narrateur|La tasse étoilée a le toc le plus petit, le juste.
-maman|Quel moment tu gardes, Mila ?
-enfant-f|Celui des trois tocs, de plus en plus vrais.
+maman|Les trois tocs étaient justes ?
+enfant-f|De plus en plus vrais, un par un.
 papa|Le chausson n'est plus dans le seau.
 narrateur|Un dernier petit toc, puis le cacao.
 enfant-f|J'ai mis l'ordre, pas la chambre.
@@ -16076,17 +16076,17 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Au campement, le seau cale le tapis, vide et sage. L'écharpe tient Mila. Le carré tient l'anse. Le soleil de souffle a des rayons, et des mains vides. Quel moment tu gardes, Mila ? Celui où mes mains n'avaient plus rien à rattraper. Le chausson est rentré sous le lit, pour de bon. Un toc, puis plus de bascule. J'ai soufflé, les mains libres. Sur le verre, la goutte a pris un rayon, sans chute. Le pied du campement ne glisse plus.</t>
+          <t>Au campement, le seau cale le tapis, vide et sage. L'écharpe tient Mila. Le carré tient l'anse. Le soleil de souffle a des rayons, et des mains vides. Tes mains n'avaient plus rien à rattraper ? Libres, pendant que je soufflais. Le chausson est rentré sous le lit, pour de bon. Un toc, puis plus de bascule. J'ai soufflé, les mains libres. Sur le verre, la goutte a pris un rayon, sans chute. Le pied du campement ne glisse plus.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, le seau cale le tapis, vide et sage. L'écharpe tient Mila. Le carré tient l'anse. Le soleil de souffle a des rayons, et des mains vides. Quel moment tu gardes, Mila ? Celui où mes mains n'avaient plus rien à rattraper. Le chausson est rentré sous le lit, pour de bon. Un toc, puis plus de bascule. J'ai soufflé, les mains libres. Sur le verre, la &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; a pris un rayon, sans chute. Le pied du campement ne glisse plus.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, le seau cale le tapis, vide et sage. L'écharpe tient Mila. Le carré tient l'anse. Le soleil de souffle a des rayons, et des mains vides. Tes mains n'avaient plus rien à rattraper ? Libres, pendant que je soufflais. Le chausson est rentré sous le lit, pour de bon. Un toc, puis plus de bascule. J'ai soufflé, les mains libres. Sur le verre, la &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; a pris un rayon, sans chute. Le pied du campement ne glisse plus.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, le seau cale le tapis, vide et sage. L'écharpe tient Mila. Le carré tient l'anse. Le soleil de souffle a des rayons, et des mains vides. Quel moment tu gardes, Mila ? Celui où mes mains n'avaient plus rien à rattraper. Le chausson est rentré sous le lit, pour de bon. Un toc, puis plus de bascule. J'ai soufflé, les mains libres. Sur le verre, la &lt;emphasis&gt;goutte&lt;/emphasis&gt; a pris un rayon, sans chute. Le pied du campement ne glisse plus.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, le seau cale le tapis, vide et sage. L'écharpe tient Mila. Le carré tient l'anse. Le soleil de souffle a des rayons, et des mains vides. Tes mains n'avaient plus rien à rattraper ? Libres, pendant que je soufflais. Le chausson est rentré sous le lit, pour de bon. Un toc, puis plus de bascule. J'ai soufflé, les mains libres. Sur le verre, la &lt;emphasis&gt;goutte&lt;/emphasis&gt; a pris un rayon, sans chute. Le pied du campement ne glisse plus.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr"/>
@@ -16228,8 +16228,8 @@
 narrateur|L'écharpe tient Mila.
 narrateur|Le carré tient l'anse.
 narrateur|Le soleil de souffle a des rayons, et des mains vides.
-maman|Quel moment tu gardes, Mila ?
-enfant-f|Celui où mes mains n'avaient plus rien à rattraper.
+maman|Tes mains n'avaient plus rien à rattraper ?
+enfant-f|Libres, pendant que je soufflais.
 papa|Le chausson est rentré sous le lit, pour de bon.
 narrateur|Un toc, puis plus de bascule.
 enfant-f|J'ai soufflé, les mains libres.
@@ -16858,17 +16858,17 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Au campement, deux soleils : le bon, et le petit à gauche. Le doudou s'assoit sous le petit, sans toucher l'anse. Le crayon a fini les deux ronds, sans se tromper. Quel moment tu gardes, Mila ? Celui où le mauvais beige a eu sa place, à part. Le carré, lui, reste sous la vraie étoile. Un toc net, du bon côté. J'ai dessiné pour ne plus mêler les deux. Sur le verre, la goutte habite le plus grand rond. Le petit rond, vide, suffit au doudou.</t>
+          <t>Au campement, deux soleils : le bon, et le petit à gauche. Le doudou s'assoit sous le petit, sans toucher l'anse. Le crayon a fini les deux ronds, sans se tromper. Le mauvais beige a eu sa place ? À part, sous son petit rond. Le carré, lui, reste sous la vraie étoile. Un toc net, du bon côté. J'ai dessiné pour ne plus mêler les deux. Sur le verre, la goutte habite le plus grand rond. Le petit rond, vide, suffit au doudou.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, deux soleils : le bon, et le petit à gauche. Le doudou s'assoit sous le petit, sans toucher l'anse. Le crayon a fini les deux ronds, sans se tromper. Quel moment tu gardes, Mila ? Celui où le mauvais beige a eu sa place, à part. Le carré, lui, reste sous la vraie étoile. Un toc net, du bon côté. J'ai dessiné pour ne plus mêler les deux. Sur le verre, la &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; habite le plus grand rond. Le petit rond, vide, suffit au doudou.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, deux soleils : le bon, et le petit à gauche. Le doudou s'assoit sous le petit, sans toucher l'anse. Le crayon a fini les deux ronds, sans se tromper. Le mauvais beige a eu sa place ? À part, sous son petit rond. Le carré, lui, reste sous la vraie étoile. Un toc net, du bon côté. J'ai dessiné pour ne plus mêler les deux. Sur le verre, la &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt; habite le plus grand rond. Le petit rond, vide, suffit au doudou.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, deux soleils : le bon, et le petit à gauche. Le doudou s'assoit sous le petit, sans toucher l'anse. Le crayon a fini les deux ronds, sans se tromper. Quel moment tu gardes, Mila ? Celui où le mauvais beige a eu sa place, à part. Le carré, lui, reste sous la vraie étoile. Un toc net, du bon côté. J'ai dessiné pour ne plus mêler les deux. Sur le verre, la &lt;emphasis&gt;goutte&lt;/emphasis&gt; habite le plus grand rond. Le petit rond, vide, suffit au doudou.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, deux soleils : le bon, et le petit à gauche. Le doudou s'assoit sous le petit, sans toucher l'anse. Le crayon a fini les deux ronds, sans se tromper. Le mauvais beige a eu sa place ? À part, sous son petit rond. Le carré, lui, reste sous la vraie étoile. Un toc net, du bon côté. J'ai dessiné pour ne plus mêler les deux. Sur le verre, la &lt;emphasis&gt;goutte&lt;/emphasis&gt; habite le plus grand rond. Le petit rond, vide, suffit au doudou.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr"/>
@@ -17009,8 +17009,8 @@
           <t>narrateur|Au campement, deux soleils : le bon, et le petit à gauche.
 narrateur|Le doudou s'assoit sous le petit, sans toucher l'anse.
 narrateur|Le crayon a fini les deux ronds, sans se tromper.
-maman|Quel moment tu gardes, Mila ?
-enfant-f|Celui où le mauvais beige a eu sa place, à part.
+maman|Le mauvais beige a eu sa place ?
+enfant-f|À part, sous son petit rond.
 papa|Le carré, lui, reste sous la vraie étoile.
 narrateur|Un toc net, du bon côté.
 enfant-f|J'ai dessiné pour ne plus mêler les deux.
@@ -17243,17 +17243,17 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Au campement, un seul rond de doigt, le bon. Le doudou, ami, n'est plus un gant. La tasse étoilée, dans le carré, a le toc franc. Quel moment tu gardes, Mila ? Celui où le doudou a eu le droit d'être lui. Le carré, lui, reste le gant de l'anse. Un toc franc, sans double beige. J'ai bu, et chacun avait son métier. Sur le verre, un seul point-goutte, sous le bon soleil. Le nid de laine, loin, est juste un nid.</t>
+          <t>Au campement, un seul rond de doigt, le bon. Le doudou, ami, n'est plus un gant. La tasse étoilée, dans le carré, a le toc franc. Le doudou a eu le droit d'être lui ? Un ami, plus un gant. Le carré, lui, reste le gant de l'anse. Un toc franc, sans double beige. J'ai bu, et chacun avait son métier. Sur le verre, un seul point-goutte, sous le bon soleil. Le nid de laine, loin, est juste un nid.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, un seul rond de doigt, le bon. Le doudou, ami, n'est plus un gant. La tasse étoilée, dans le carré, a le toc franc. Quel moment tu gardes, Mila ? Celui où le doudou a eu le droit d'être lui. Le carré, lui, reste le gant de l'anse. Un toc franc, sans double beige. J'ai bu, et chacun avait son métier. Sur le verre, un seul point-&lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt;, sous le bon soleil. Le nid de laine, loin, est juste un nid.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, un seul rond de doigt, le bon. Le doudou, ami, n'est plus un gant. La tasse étoilée, dans le carré, a le toc franc. Le doudou a eu le droit d'être lui ? Un ami, plus un gant. Le carré, lui, reste le gant de l'anse. Un toc franc, sans double beige. J'ai bu, et chacun avait son métier. Sur le verre, un seul point-&lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt;, sous le bon soleil. Le nid de laine, loin, est juste un nid.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, un seul rond de doigt, le bon. Le doudou, ami, n'est plus un gant. La tasse étoilée, dans le carré, a le toc franc. Quel moment tu gardes, Mila ? Celui où le doudou a eu le droit d'être lui. Le carré, lui, reste le gant de l'anse. Un toc franc, sans double beige. J'ai bu, et chacun avait son métier. Sur le verre, un seul point-&lt;emphasis&gt;goutte&lt;/emphasis&gt;, sous le bon soleil. Le nid de laine, loin, est juste un nid.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, un seul rond de doigt, le bon. Le doudou, ami, n'est plus un gant. La tasse étoilée, dans le carré, a le toc franc. Le doudou a eu le droit d'être lui ? Un ami, plus un gant. Le carré, lui, reste le gant de l'anse. Un toc franc, sans double beige. J'ai bu, et chacun avait son métier. Sur le verre, un seul point-&lt;emphasis&gt;goutte&lt;/emphasis&gt;, sous le bon soleil. Le nid de laine, loin, est juste un nid.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr"/>
@@ -17394,8 +17394,8 @@
           <t>narrateur|Au campement, un seul rond de doigt, le bon.
 narrateur|Le doudou, ami, n'est plus un gant.
 narrateur|La tasse étoilée, dans le carré, a le toc franc.
-maman|Quel moment tu gardes, Mila ?
-enfant-f|Celui où le doudou a eu le droit d'être lui.
+maman|Le doudou a eu le droit d'être lui ?
+enfant-f|Un ami, plus un gant.
 papa|Le carré, lui, reste le gant de l'anse.
 narrateur|Un toc franc, sans double beige.
 enfant-f|J'ai bu, et chacun avait son métier.
@@ -17634,17 +17634,17 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Au campement, trois chauds, un sourire de goutte. L'étoile bleue a sa fenêtre. Le doudou, son petit rond. L'écharpe sent le cacao, et un peu la chambre. Quel moment tu gardes, Mila ? Celui où personne n'était sur les pieds de personne. La tasse étoilée fume à peine, juste assez. Un toc, puis le sourire qui ne glisse plus. J'ai soufflé pour le grand, et laissé le petit. Sur le verre, la goutte du début est un sourire, en bas. Le campement tient, plein et clair, jusqu'à Nina.</t>
+          <t>Au campement, trois chauds, un sourire de goutte. L'étoile bleue a sa fenêtre. Le doudou, son petit rond. L'écharpe sent le cacao, et un peu la chambre. Personne sur les pieds de personne ? Trois places, et le verre à nous. La tasse étoilée fume à peine, juste assez. Un toc, puis le sourire qui ne glisse plus. J'ai soufflé pour le grand, et laissé le petit. Sur le verre, la goutte du début est un sourire, en bas. Le campement tient, plein et clair, jusqu'à Nina.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, trois chauds, un sourire de &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt;. L'étoile bleue a sa fenêtre. Le doudou, son petit rond. L'écharpe sent le cacao, et un peu la chambre. Quel moment tu gardes, Mila ? Celui où personne n'était sur les pieds de personne. La tasse étoilée fume à peine, juste assez. Un toc, puis le sourire qui ne glisse plus. J'ai soufflé pour le grand, et laissé le petit. Sur le verre, la goutte du début est un sourire, en bas. Le campement tient, plein et clair, jusqu'à Nina.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au campement, trois chauds, un sourire de &lt;emphasis level="moderate"&gt;goutte&lt;/emphasis&gt;. L'étoile bleue a sa fenêtre. Le doudou, son petit rond. L'écharpe sent le cacao, et un peu la chambre. Personne sur les pieds de personne ? Trois places, et le verre à nous. La tasse étoilée fume à peine, juste assez. Un toc, puis le sourire qui ne glisse plus. J'ai soufflé pour le grand, et laissé le petit. Sur le verre, la goutte du début est un sourire, en bas. Le campement tient, plein et clair, jusqu'à Nina.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, trois chauds, un sourire de &lt;emphasis&gt;goutte&lt;/emphasis&gt;. L'étoile bleue a sa fenêtre. Le doudou, son petit rond. L'écharpe sent le cacao, et un peu la chambre. Quel moment tu gardes, Mila ? Celui où personne n'était sur les pieds de personne. La tasse étoilée fume à peine, juste assez. Un toc, puis le sourire qui ne glisse plus. J'ai soufflé pour le grand, et laissé le petit. Sur le verre, la goutte du début est un sourire, en bas. Le campement tient, plein et clair, jusqu'à Nina.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au campement, trois chauds, un sourire de &lt;emphasis&gt;goutte&lt;/emphasis&gt;. L'étoile bleue a sa fenêtre. Le doudou, son petit rond. L'écharpe sent le cacao, et un peu la chambre. Personne sur les pieds de personne ? Trois places, et le verre à nous. La tasse étoilée fume à peine, juste assez. Un toc, puis le sourire qui ne glisse plus. J'ai soufflé pour le grand, et laissé le petit. Sur le verre, la goutte du début est un sourire, en bas. Le campement tient, plein et clair, jusqu'à Nina.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr"/>
@@ -17786,8 +17786,8 @@
 narrateur|L'étoile bleue a sa fenêtre.
 narrateur|Le doudou, son petit rond.
 narrateur|L'écharpe sent le cacao, et un peu la chambre.
-maman|Quel moment tu gardes, Mila ?
-enfant-f|Celui où personne n'était sur les pieds de personne.
+maman|Personne sur les pieds de personne ?
+enfant-f|Trois places, et le verre à nous.
 papa|La tasse étoilée fume à peine, juste assez.
 narrateur|Un toc, puis le sourire qui ne glisse plus.
 enfant-f|J'ai soufflé pour le grand, et laissé le petit.
@@ -17818,7 +17818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17938,6 +17938,13 @@
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>